<commit_message>
Daily rebuild Tue 05/26/2026  9:06:48.00
</commit_message>
<xml_diff>
--- a/generated/Fleet Pipeline/BDM_Fleet_Pipeline_Report.xlsx
+++ b/generated/Fleet Pipeline/BDM_Fleet_Pipeline_Report.xlsx
@@ -546,10 +546,10 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>5489248.23</v>
+        <v>5414310.25</v>
       </c>
     </row>
     <row r="7">
@@ -36040,7 +36040,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M66"/>
+  <dimension ref="A1:M65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -36433,12 +36433,12 @@
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>268473189456</t>
+          <t>259436020243</t>
         </is>
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>GGM TRANSPORT LLC</t>
+          <t>AVI TRANSPORTATION SERVICES INC</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
@@ -36447,7 +36447,7 @@
         </is>
       </c>
       <c r="D7" s="10" t="n">
-        <v>74937.98</v>
+        <v>55880.12</v>
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
@@ -36459,31 +36459,31 @@
       </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
-          <t>MI</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="H7" s="9" t="inlineStr">
         <is>
-          <t>Resolute Insurance Group LLC</t>
+          <t>American Fleet Insurance</t>
         </is>
       </c>
       <c r="I7" s="9" t="inlineStr">
         <is>
-          <t>Colton Duty</t>
+          <t>Justin Feaster</t>
         </is>
       </c>
       <c r="J7" s="9" t="inlineStr">
         <is>
-          <t>04/27/2026</t>
+          <t>06/07/2025</t>
         </is>
       </c>
       <c r="K7" s="9" t="inlineStr">
         <is>
-          <t>01/28/2026</t>
+          <t>01/05/2026</t>
         </is>
       </c>
       <c r="L7" s="9" t="n">
-        <v>3716900</v>
+        <v>3221114</v>
       </c>
       <c r="M7" s="9" t="inlineStr">
         <is>
@@ -36494,12 +36494,12 @@
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>259436020243</t>
+          <t>269901996335</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>AVI TRANSPORTATION SERVICES INC</t>
+          <t>ERIC CHAIDEZ</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
@@ -36508,7 +36508,7 @@
         </is>
       </c>
       <c r="D8" s="8" t="n">
-        <v>55880.12</v>
+        <v>49487.45</v>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
@@ -36520,31 +36520,31 @@
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>American Fleet Insurance</t>
+          <t>AMC Agents LLC</t>
         </is>
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
-          <t>Justin Feaster</t>
+          <t>Andres Piedrahita</t>
         </is>
       </c>
       <c r="J8" s="7" t="inlineStr">
         <is>
-          <t>06/07/2025</t>
+          <t>05/08/2026</t>
         </is>
       </c>
       <c r="K8" s="7" t="inlineStr">
         <is>
-          <t>01/05/2026</t>
+          <t>02/08/2026</t>
         </is>
       </c>
       <c r="L8" s="7" t="n">
-        <v>3221114</v>
+        <v>1936547</v>
       </c>
       <c r="M8" s="7" t="inlineStr">
         <is>
@@ -36555,12 +36555,12 @@
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>269901996335</t>
+          <t>264118066290</t>
         </is>
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>ERIC CHAIDEZ</t>
+          <t>ROAD TRUCKS SOLUTIONS CORP</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
@@ -36569,19 +36569,19 @@
         </is>
       </c>
       <c r="D9" s="10" t="n">
-        <v>49487.45</v>
+        <v>5924.6</v>
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F9" s="9" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="H9" s="9" t="inlineStr">
@@ -36596,16 +36596,16 @@
       </c>
       <c r="J9" s="9" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>06/30/2026</t>
         </is>
       </c>
       <c r="K9" s="9" t="inlineStr">
         <is>
-          <t>02/08/2026</t>
+          <t>03/31/2026</t>
         </is>
       </c>
       <c r="L9" s="9" t="n">
-        <v>1936547</v>
+        <v>2468970</v>
       </c>
       <c r="M9" s="9" t="inlineStr">
         <is>
@@ -36616,29 +36616,29 @@
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>264118066290</t>
+          <t>265739244226</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>ROAD TRUCKS SOLUTIONS CORP</t>
+          <t>N&amp;J BROS BREAD DISTRIBUTIONS INC</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Quoted</t>
+          <t>Submitted</t>
         </is>
       </c>
       <c r="D10" s="8" t="n">
-        <v>5924.6</v>
+        <v>725914.11</v>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F10" s="7" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
@@ -36647,26 +36647,26 @@
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>AMC Agents LLC</t>
+          <t>American Fleet Insurance</t>
         </is>
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>Andres Piedrahita</t>
+          <t>Justin Feaster</t>
         </is>
       </c>
       <c r="J10" s="7" t="inlineStr">
         <is>
-          <t>06/30/2026</t>
+          <t>02/12/2026</t>
         </is>
       </c>
       <c r="K10" s="7" t="inlineStr">
         <is>
-          <t>03/31/2026</t>
+          <t>02/11/2026</t>
         </is>
       </c>
       <c r="L10" s="7" t="n">
-        <v>2468970</v>
+        <v>3935916</v>
       </c>
       <c r="M10" s="7" t="inlineStr">
         <is>
@@ -36677,12 +36677,12 @@
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>265739244226</t>
+          <t>260572353010</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>N&amp;J BROS BREAD DISTRIBUTIONS INC</t>
+          <t>CARWAY LOGISTICS INC</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
@@ -36691,7 +36691,7 @@
         </is>
       </c>
       <c r="D11" s="10" t="n">
-        <v>725914.11</v>
+        <v>675272.02</v>
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
@@ -36699,35 +36699,35 @@
         </is>
       </c>
       <c r="F11" s="9" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t>FL</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="H11" s="9" t="inlineStr">
         <is>
-          <t>American Fleet Insurance</t>
+          <t>InsurNorth Corp</t>
         </is>
       </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t>Justin Feaster</t>
+          <t>Ali Boyko</t>
         </is>
       </c>
       <c r="J11" s="9" t="inlineStr">
         <is>
-          <t>02/12/2026</t>
+          <t>03/25/2026</t>
         </is>
       </c>
       <c r="K11" s="9" t="inlineStr">
         <is>
-          <t>02/11/2026</t>
+          <t>03/24/2026</t>
         </is>
       </c>
       <c r="L11" s="9" t="n">
-        <v>3935916</v>
+        <v>4120945</v>
       </c>
       <c r="M11" s="9" t="inlineStr">
         <is>
@@ -36738,12 +36738,12 @@
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>260572353010</t>
+          <t>260829434198</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>CARWAY LOGISTICS INC</t>
+          <t>FNI LOGISTICS INC</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
@@ -36752,7 +36752,7 @@
         </is>
       </c>
       <c r="D12" s="8" t="n">
-        <v>675272.02</v>
+        <v>626500.5699999999</v>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
@@ -36760,7 +36760,7 @@
         </is>
       </c>
       <c r="F12" s="7" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
@@ -36769,12 +36769,12 @@
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>InsurNorth Corp</t>
+          <t>Lone Star Direct Insurance Agency LLC</t>
         </is>
       </c>
       <c r="I12" s="7" t="inlineStr">
         <is>
-          <t>Ali Boyko</t>
+          <t>Zafarjon Khonkeldiev</t>
         </is>
       </c>
       <c r="J12" s="7" t="inlineStr">
@@ -36784,11 +36784,11 @@
       </c>
       <c r="K12" s="7" t="inlineStr">
         <is>
-          <t>03/24/2026</t>
+          <t>03/12/2026</t>
         </is>
       </c>
       <c r="L12" s="7" t="n">
-        <v>4120945</v>
+        <v>3538162</v>
       </c>
       <c r="M12" s="7" t="inlineStr">
         <is>
@@ -36799,12 +36799,12 @@
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
         <is>
-          <t>260829434198</t>
+          <t>260668840119</t>
         </is>
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>FNI LOGISTICS INC</t>
+          <t>TURBO TRANSPORT LLC</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
@@ -36813,7 +36813,7 @@
         </is>
       </c>
       <c r="D13" s="10" t="n">
-        <v>626500.5699999999</v>
+        <v>397880.13</v>
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
@@ -36821,35 +36821,35 @@
         </is>
       </c>
       <c r="F13" s="9" t="n">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="H13" s="9" t="inlineStr">
         <is>
-          <t>Lone Star Direct Insurance Agency LLC</t>
+          <t>American Fleet Insurance</t>
         </is>
       </c>
       <c r="I13" s="9" t="inlineStr">
         <is>
-          <t>Zafarjon Khonkeldiev</t>
+          <t>Justin Feaster</t>
         </is>
       </c>
       <c r="J13" s="9" t="inlineStr">
         <is>
-          <t>03/25/2026</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="K13" s="9" t="inlineStr">
         <is>
-          <t>03/12/2026</t>
+          <t>02/02/2026</t>
         </is>
       </c>
       <c r="L13" s="9" t="n">
-        <v>3538162</v>
+        <v>3413378</v>
       </c>
       <c r="M13" s="9" t="inlineStr">
         <is>
@@ -36860,12 +36860,12 @@
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>260668840119</t>
+          <t>261563637238</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>TURBO TRANSPORT LLC</t>
+          <t>C2C DISPATCH LLC</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
@@ -36874,7 +36874,7 @@
         </is>
       </c>
       <c r="D14" s="8" t="n">
-        <v>397880.13</v>
+        <v>375803.34</v>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
@@ -36882,35 +36882,35 @@
         </is>
       </c>
       <c r="F14" s="7" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>American Fleet Insurance</t>
+          <t>Resolute Insurance Group LLC</t>
         </is>
       </c>
       <c r="I14" s="7" t="inlineStr">
         <is>
-          <t>Justin Feaster</t>
+          <t>Josh Connor</t>
         </is>
       </c>
       <c r="J14" s="7" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>02/07/2026</t>
         </is>
       </c>
       <c r="K14" s="7" t="inlineStr">
         <is>
-          <t>02/02/2026</t>
+          <t>01/28/2026</t>
         </is>
       </c>
       <c r="L14" s="7" t="n">
-        <v>3413378</v>
+        <v>4177194</v>
       </c>
       <c r="M14" s="7" t="inlineStr">
         <is>
@@ -36921,12 +36921,12 @@
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>261563637238</t>
+          <t>266591984430</t>
         </is>
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>C2C DISPATCH LLC</t>
+          <t>24 7 LOGISTICS LLC</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
@@ -36935,7 +36935,7 @@
         </is>
       </c>
       <c r="D15" s="10" t="n">
-        <v>375803.34</v>
+        <v>199190</v>
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
@@ -36947,31 +36947,31 @@
       </c>
       <c r="G15" s="9" t="inlineStr">
         <is>
-          <t>FL</t>
+          <t>MN</t>
         </is>
       </c>
       <c r="H15" s="9" t="inlineStr">
         <is>
-          <t>Resolute Insurance Group LLC</t>
+          <t>Protectgo Services LLC</t>
         </is>
       </c>
       <c r="I15" s="9" t="inlineStr">
         <is>
-          <t>Josh Connor</t>
+          <t>Christopher Salazar</t>
         </is>
       </c>
       <c r="J15" s="9" t="inlineStr">
         <is>
-          <t>02/07/2026</t>
+          <t>02/12/2026</t>
         </is>
       </c>
       <c r="K15" s="9" t="inlineStr">
         <is>
-          <t>01/28/2026</t>
+          <t>02/10/2026</t>
         </is>
       </c>
       <c r="L15" s="9" t="n">
-        <v>4177194</v>
+        <v>3227451</v>
       </c>
       <c r="M15" s="9" t="inlineStr">
         <is>
@@ -36982,12 +36982,12 @@
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>266591984430</t>
+          <t>263495807059</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>24 7 LOGISTICS LLC</t>
+          <t>MVL TRUCKING INC</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
@@ -36996,7 +36996,7 @@
         </is>
       </c>
       <c r="D16" s="8" t="n">
-        <v>199190</v>
+        <v>181550.84</v>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
@@ -37004,35 +37004,35 @@
         </is>
       </c>
       <c r="F16" s="7" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>MN</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>Protectgo Services LLC</t>
+          <t>AMC Agents LLC</t>
         </is>
       </c>
       <c r="I16" s="7" t="inlineStr">
         <is>
-          <t>Christopher Salazar</t>
+          <t>Carlos Ochoa</t>
         </is>
       </c>
       <c r="J16" s="7" t="inlineStr">
         <is>
-          <t>02/12/2026</t>
+          <t>04/08/2026</t>
         </is>
       </c>
       <c r="K16" s="7" t="inlineStr">
         <is>
-          <t>02/10/2026</t>
+          <t>03/11/2026</t>
         </is>
       </c>
       <c r="L16" s="7" t="n">
-        <v>3227451</v>
+        <v>2867469</v>
       </c>
       <c r="M16" s="7" t="inlineStr">
         <is>
@@ -37043,12 +37043,12 @@
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>263495807059</t>
+          <t>265750278915</t>
         </is>
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>MVL TRUCKING INC</t>
+          <t>NICE TRANS LLC</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
@@ -37057,7 +37057,7 @@
         </is>
       </c>
       <c r="D17" s="10" t="n">
-        <v>181550.84</v>
+        <v>162388.17</v>
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
@@ -37065,35 +37065,35 @@
         </is>
       </c>
       <c r="F17" s="9" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="G17" s="9" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="H17" s="9" t="inlineStr">
         <is>
-          <t>AMC Agents LLC</t>
+          <t>American Fleet Insurance</t>
         </is>
       </c>
       <c r="I17" s="9" t="inlineStr">
         <is>
-          <t>Carlos Ochoa</t>
+          <t>Justin Feaster</t>
         </is>
       </c>
       <c r="J17" s="9" t="inlineStr">
         <is>
-          <t>04/08/2026</t>
+          <t>02/01/2026</t>
         </is>
       </c>
       <c r="K17" s="9" t="inlineStr">
         <is>
-          <t>03/11/2026</t>
+          <t>01/12/2026</t>
         </is>
       </c>
       <c r="L17" s="9" t="n">
-        <v>2867469</v>
+        <v>3209545</v>
       </c>
       <c r="M17" s="9" t="inlineStr">
         <is>
@@ -37104,12 +37104,12 @@
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>265750278915</t>
+          <t>269483884540</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>NICE TRANS LLC</t>
+          <t>LACOH TRANSPORT INC</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
@@ -37118,7 +37118,7 @@
         </is>
       </c>
       <c r="D18" s="8" t="n">
-        <v>162388.17</v>
+        <v>132719.3</v>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
@@ -37126,11 +37126,11 @@
         </is>
       </c>
       <c r="F18" s="7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="H18" s="7" t="inlineStr">
@@ -37145,16 +37145,16 @@
       </c>
       <c r="J18" s="7" t="inlineStr">
         <is>
-          <t>02/01/2026</t>
+          <t>01/20/2026</t>
         </is>
       </c>
       <c r="K18" s="7" t="inlineStr">
         <is>
-          <t>01/12/2026</t>
+          <t>01/09/2026</t>
         </is>
       </c>
       <c r="L18" s="7" t="n">
-        <v>3209545</v>
+        <v>991231</v>
       </c>
       <c r="M18" s="7" t="inlineStr">
         <is>
@@ -37165,12 +37165,12 @@
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>269483884540</t>
+          <t>267262775539</t>
         </is>
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>LACOH TRANSPORT INC</t>
+          <t>YO YO TRANSPORT LLC</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
@@ -37179,7 +37179,7 @@
         </is>
       </c>
       <c r="D19" s="10" t="n">
-        <v>132719.3</v>
+        <v>123862.69</v>
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
@@ -37187,35 +37187,35 @@
         </is>
       </c>
       <c r="F19" s="9" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G19" s="9" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="H19" s="9" t="inlineStr">
         <is>
-          <t>American Fleet Insurance</t>
+          <t>Resolute Insurance Group LLC</t>
         </is>
       </c>
       <c r="I19" s="9" t="inlineStr">
         <is>
-          <t>Justin Feaster</t>
+          <t>Josh Connor</t>
         </is>
       </c>
       <c r="J19" s="9" t="inlineStr">
         <is>
-          <t>01/20/2026</t>
+          <t>02/06/2026</t>
         </is>
       </c>
       <c r="K19" s="9" t="inlineStr">
         <is>
-          <t>01/09/2026</t>
+          <t>01/27/2026</t>
         </is>
       </c>
       <c r="L19" s="9" t="n">
-        <v>991231</v>
+        <v>3789738</v>
       </c>
       <c r="M19" s="9" t="inlineStr">
         <is>
@@ -37226,12 +37226,12 @@
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>267262775539</t>
+          <t>264425523628</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>YO YO TRANSPORT LLC</t>
+          <t>ES RELOCATION SERVICES INC</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
@@ -37240,7 +37240,7 @@
         </is>
       </c>
       <c r="D20" s="8" t="n">
-        <v>123862.69</v>
+        <v>108905.16</v>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
@@ -37248,35 +37248,35 @@
         </is>
       </c>
       <c r="F20" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="H20" s="7" t="inlineStr">
         <is>
-          <t>Resolute Insurance Group LLC</t>
+          <t>American Fleet Insurance</t>
         </is>
       </c>
       <c r="I20" s="7" t="inlineStr">
         <is>
-          <t>Josh Connor</t>
+          <t>Justin Feaster</t>
         </is>
       </c>
       <c r="J20" s="7" t="inlineStr">
         <is>
+          <t>02/07/2026</t>
+        </is>
+      </c>
+      <c r="K20" s="7" t="inlineStr">
+        <is>
           <t>02/06/2026</t>
         </is>
       </c>
-      <c r="K20" s="7" t="inlineStr">
-        <is>
-          <t>01/27/2026</t>
-        </is>
-      </c>
       <c r="L20" s="7" t="n">
-        <v>3789738</v>
+        <v>4086660</v>
       </c>
       <c r="M20" s="7" t="inlineStr">
         <is>
@@ -37287,12 +37287,12 @@
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>264425523628</t>
+          <t>261924516505</t>
         </is>
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>ES RELOCATION SERVICES INC</t>
+          <t>D&amp;D BROS INC</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
@@ -37301,11 +37301,11 @@
         </is>
       </c>
       <c r="D21" s="10" t="n">
-        <v>108905.16</v>
+        <v>93067.12</v>
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F21" s="9" t="n">
@@ -37313,31 +37313,31 @@
       </c>
       <c r="G21" s="9" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="H21" s="9" t="inlineStr">
         <is>
-          <t>American Fleet Insurance</t>
+          <t>Resolute Insurance Group LLC</t>
         </is>
       </c>
       <c r="I21" s="9" t="inlineStr">
         <is>
-          <t>Justin Feaster</t>
+          <t>Josh Connor</t>
         </is>
       </c>
       <c r="J21" s="9" t="inlineStr">
         <is>
-          <t>02/07/2026</t>
+          <t>01/26/2026</t>
         </is>
       </c>
       <c r="K21" s="9" t="inlineStr">
         <is>
-          <t>02/06/2026</t>
+          <t>01/15/2026</t>
         </is>
       </c>
       <c r="L21" s="9" t="n">
-        <v>4086660</v>
+        <v>3735644</v>
       </c>
       <c r="M21" s="9" t="inlineStr">
         <is>
@@ -37348,12 +37348,12 @@
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>261924516505</t>
+          <t>265357815377</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>D&amp;D BROS INC</t>
+          <t>AM TRUCK ENTERPRISES LLC</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
@@ -37362,7 +37362,7 @@
         </is>
       </c>
       <c r="D22" s="8" t="n">
-        <v>93067.12</v>
+        <v>68282.13</v>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
@@ -37374,7 +37374,7 @@
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="H22" s="7" t="inlineStr">
@@ -37389,16 +37389,16 @@
       </c>
       <c r="J22" s="7" t="inlineStr">
         <is>
-          <t>01/26/2026</t>
+          <t>03/17/2026</t>
         </is>
       </c>
       <c r="K22" s="7" t="inlineStr">
         <is>
-          <t>01/15/2026</t>
+          <t>02/24/2026</t>
         </is>
       </c>
       <c r="L22" s="7" t="n">
-        <v>3735644</v>
+        <v>2887715</v>
       </c>
       <c r="M22" s="7" t="inlineStr">
         <is>
@@ -37409,12 +37409,12 @@
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>265357815377</t>
+          <t>264971243711</t>
         </is>
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>AM TRUCK ENTERPRISES LLC</t>
+          <t>ADVANCED FREIGHT LLC</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
@@ -37423,7 +37423,7 @@
         </is>
       </c>
       <c r="D23" s="10" t="n">
-        <v>68282.13</v>
+        <v>55742.32</v>
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
@@ -37435,31 +37435,31 @@
       </c>
       <c r="G23" s="9" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>OR</t>
         </is>
       </c>
       <c r="H23" s="9" t="inlineStr">
         <is>
-          <t>Resolute Insurance Group LLC</t>
+          <t>InsurNorth Corp</t>
         </is>
       </c>
       <c r="I23" s="9" t="inlineStr">
         <is>
-          <t>Josh Connor</t>
+          <t>Ali Boyko</t>
         </is>
       </c>
       <c r="J23" s="9" t="inlineStr">
         <is>
-          <t>03/17/2026</t>
+          <t>03/15/2026</t>
         </is>
       </c>
       <c r="K23" s="9" t="inlineStr">
         <is>
-          <t>02/24/2026</t>
+          <t>03/11/2026</t>
         </is>
       </c>
       <c r="L23" s="9" t="n">
-        <v>2887715</v>
+        <v>3478431</v>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
@@ -37470,12 +37470,12 @@
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>264971243711</t>
+          <t>268723958142</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>ADVANCED FREIGHT LLC</t>
+          <t>NOAH STAR TRANSPORT LLC</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
@@ -37484,7 +37484,7 @@
         </is>
       </c>
       <c r="D24" s="8" t="n">
-        <v>55742.32</v>
+        <v>53437.27</v>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
@@ -37496,31 +37496,31 @@
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>OR</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="H24" s="7" t="inlineStr">
         <is>
-          <t>InsurNorth Corp</t>
+          <t>American Fleet Insurance</t>
         </is>
       </c>
       <c r="I24" s="7" t="inlineStr">
         <is>
-          <t>Ali Boyko</t>
+          <t>Justin Feaster</t>
         </is>
       </c>
       <c r="J24" s="7" t="inlineStr">
         <is>
-          <t>03/15/2026</t>
+          <t>02/10/2026</t>
         </is>
       </c>
       <c r="K24" s="7" t="inlineStr">
         <is>
-          <t>03/11/2026</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="L24" s="7" t="n">
-        <v>3478431</v>
+        <v>3402347</v>
       </c>
       <c r="M24" s="7" t="inlineStr">
         <is>
@@ -37531,12 +37531,12 @@
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>268723958142</t>
+          <t>259074596391</t>
         </is>
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>NOAH STAR TRANSPORT LLC</t>
+          <t>GOM TRUCKING LLC</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
@@ -37545,7 +37545,7 @@
         </is>
       </c>
       <c r="D25" s="10" t="n">
-        <v>53437.27</v>
+        <v>50251.92</v>
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
@@ -37562,42 +37562,42 @@
       </c>
       <c r="H25" s="9" t="inlineStr">
         <is>
-          <t>American Fleet Insurance</t>
+          <t>AMC Agents LLC</t>
         </is>
       </c>
       <c r="I25" s="9" t="inlineStr">
         <is>
-          <t>Justin Feaster</t>
+          <t>Andres Piedrahita</t>
         </is>
       </c>
       <c r="J25" s="9" t="inlineStr">
         <is>
-          <t>02/10/2026</t>
+          <t>07/22/2025</t>
         </is>
       </c>
       <c r="K25" s="9" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>02/27/2026</t>
         </is>
       </c>
       <c r="L25" s="9" t="n">
-        <v>3402347</v>
+        <v>4366449</v>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>eld_only</t>
+          <t>dash_cam_dual_ai_connected</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>259074596391</t>
+          <t>261309140377</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>GOM TRUCKING LLC</t>
+          <t>KANDAHAR LOGISTICS LLC</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
@@ -37606,7 +37606,7 @@
         </is>
       </c>
       <c r="D26" s="8" t="n">
-        <v>50251.92</v>
+        <v>46366</v>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
@@ -37618,47 +37618,47 @@
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="H26" s="7" t="inlineStr">
         <is>
-          <t>AMC Agents LLC</t>
+          <t>InsurNorth Corp</t>
         </is>
       </c>
       <c r="I26" s="7" t="inlineStr">
         <is>
-          <t>Andres Piedrahita</t>
+          <t>Mark Fabyanchuk</t>
         </is>
       </c>
       <c r="J26" s="7" t="inlineStr">
         <is>
-          <t>07/22/2025</t>
+          <t>01/29/2026</t>
         </is>
       </c>
       <c r="K26" s="7" t="inlineStr">
         <is>
-          <t>02/27/2026</t>
+          <t>01/28/2026</t>
         </is>
       </c>
       <c r="L26" s="7" t="n">
-        <v>4366449</v>
+        <v>3553420</v>
       </c>
       <c r="M26" s="7" t="inlineStr">
         <is>
-          <t>dash_cam_dual_ai_connected</t>
+          <t>eld_only</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>261309140377</t>
+          <t>262451035072</t>
         </is>
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>KANDAHAR LOGISTICS LLC</t>
+          <t>EZ TRANSPORT AND LOGISTICS LLC</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
@@ -37667,43 +37667,43 @@
         </is>
       </c>
       <c r="D27" s="10" t="n">
-        <v>46366</v>
+        <v>21030</v>
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F27" s="9" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="G27" s="9" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>NC</t>
         </is>
       </c>
       <c r="H27" s="9" t="inlineStr">
         <is>
-          <t>InsurNorth Corp</t>
+          <t>Resolute Insurance Group LLC</t>
         </is>
       </c>
       <c r="I27" s="9" t="inlineStr">
         <is>
-          <t>Mark Fabyanchuk</t>
+          <t>Josh Connor</t>
         </is>
       </c>
       <c r="J27" s="9" t="inlineStr">
         <is>
-          <t>01/29/2026</t>
+          <t>02/10/2026</t>
         </is>
       </c>
       <c r="K27" s="9" t="inlineStr">
         <is>
-          <t>01/28/2026</t>
+          <t>01/12/2026</t>
         </is>
       </c>
       <c r="L27" s="9" t="n">
-        <v>3553420</v>
+        <v>3716733</v>
       </c>
       <c r="M27" s="9" t="inlineStr">
         <is>
@@ -37714,12 +37714,12 @@
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>262451035072</t>
+          <t>262608227935</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>EZ TRANSPORT AND LOGISTICS LLC</t>
+          <t>S L G TRANSPORTATION SERVICE LLC</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
@@ -37728,7 +37728,7 @@
         </is>
       </c>
       <c r="D28" s="8" t="n">
-        <v>21030</v>
+        <v>20275.14</v>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
@@ -37736,51 +37736,51 @@
         </is>
       </c>
       <c r="F28" s="7" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="H28" s="7" t="inlineStr">
         <is>
-          <t>Resolute Insurance Group LLC</t>
+          <t>InsurNorth Corp</t>
         </is>
       </c>
       <c r="I28" s="7" t="inlineStr">
         <is>
-          <t>Josh Connor</t>
+          <t>Mark Fabyanchuk</t>
         </is>
       </c>
       <c r="J28" s="7" t="inlineStr">
         <is>
-          <t>02/10/2026</t>
+          <t>03/28/2026</t>
         </is>
       </c>
       <c r="K28" s="7" t="inlineStr">
         <is>
-          <t>01/12/2026</t>
+          <t>03/16/2026</t>
         </is>
       </c>
       <c r="L28" s="7" t="n">
-        <v>3716733</v>
+        <v>1126023</v>
       </c>
       <c r="M28" s="7" t="inlineStr">
         <is>
-          <t>eld_only</t>
+          <t>none</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>262608227935</t>
+          <t>262593756007</t>
         </is>
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>S L G TRANSPORTATION SERVICE LLC</t>
+          <t>OGUNS TRUCKING LLC</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
@@ -37789,7 +37789,7 @@
         </is>
       </c>
       <c r="D29" s="10" t="n">
-        <v>20275.14</v>
+        <v>17633.03</v>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
@@ -37797,35 +37797,35 @@
         </is>
       </c>
       <c r="F29" s="9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G29" s="9" t="inlineStr">
         <is>
-          <t>FL</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="H29" s="9" t="inlineStr">
         <is>
-          <t>InsurNorth Corp</t>
+          <t>Xgen Insurance Group LLC</t>
         </is>
       </c>
       <c r="I29" s="9" t="inlineStr">
         <is>
-          <t>Mark Fabyanchuk</t>
+          <t>Jaxon Alley</t>
         </is>
       </c>
       <c r="J29" s="9" t="inlineStr">
         <is>
-          <t>03/28/2026</t>
+          <t>03/19/2026</t>
         </is>
       </c>
       <c r="K29" s="9" t="inlineStr">
         <is>
-          <t>03/16/2026</t>
+          <t>03/13/2026</t>
         </is>
       </c>
       <c r="L29" s="9" t="n">
-        <v>1126023</v>
+        <v>4193710</v>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
@@ -37836,12 +37836,12 @@
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>262593756007</t>
+          <t>260117641052</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>OGUNS TRUCKING LLC</t>
+          <t>ABDIFATAH HASSAN</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
@@ -37850,7 +37850,7 @@
         </is>
       </c>
       <c r="D30" s="8" t="n">
-        <v>17633.03</v>
+        <v>10201</v>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
@@ -37858,36 +37858,34 @@
         </is>
       </c>
       <c r="F30" s="7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>MN</t>
         </is>
       </c>
       <c r="H30" s="7" t="inlineStr">
         <is>
-          <t>Xgen Insurance Group LLC</t>
+          <t>Connect Insurance Agency, Inc.</t>
         </is>
       </c>
       <c r="I30" s="7" t="inlineStr">
         <is>
-          <t>Jaxon Alley</t>
+          <t>Jeremy Huddleston</t>
         </is>
       </c>
       <c r="J30" s="7" t="inlineStr">
         <is>
-          <t>03/19/2026</t>
+          <t>01/29/2026</t>
         </is>
       </c>
       <c r="K30" s="7" t="inlineStr">
         <is>
-          <t>03/13/2026</t>
-        </is>
-      </c>
-      <c r="L30" s="7" t="n">
-        <v>4193710</v>
-      </c>
+          <t>01/28/2026</t>
+        </is>
+      </c>
+      <c r="L30" s="7" t="inlineStr"/>
       <c r="M30" s="7" t="inlineStr">
         <is>
           <t>none</t>
@@ -37897,12 +37895,12 @@
     <row r="31">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>260117641052</t>
+          <t>265970971382</t>
         </is>
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>ABDIFATAH HASSAN</t>
+          <t>Golden Axle Freightways LLC</t>
         </is>
       </c>
       <c r="C31" s="9" t="inlineStr">
@@ -37911,7 +37909,7 @@
         </is>
       </c>
       <c r="D31" s="10" t="n">
-        <v>10201</v>
+        <v>6643</v>
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
@@ -37919,31 +37917,31 @@
         </is>
       </c>
       <c r="F31" s="9" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G31" s="9" t="inlineStr">
         <is>
-          <t>MN</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="H31" s="9" t="inlineStr">
         <is>
-          <t>Connect Insurance Agency, Inc.</t>
+          <t>AMC Agents LLC</t>
         </is>
       </c>
       <c r="I31" s="9" t="inlineStr">
         <is>
-          <t>Jeremy Huddleston</t>
+          <t>Andres Piedrahita</t>
         </is>
       </c>
       <c r="J31" s="9" t="inlineStr">
         <is>
-          <t>01/29/2026</t>
+          <t>01/16/2026</t>
         </is>
       </c>
       <c r="K31" s="9" t="inlineStr">
         <is>
-          <t>01/28/2026</t>
+          <t>01/12/2026</t>
         </is>
       </c>
       <c r="L31" s="9" t="inlineStr"/>
@@ -37956,12 +37954,12 @@
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>265970971382</t>
+          <t>264034845083</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>Golden Axle Freightways LLC</t>
+          <t>ARUMA TRANSPORT LLC</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
@@ -37970,7 +37968,7 @@
         </is>
       </c>
       <c r="D32" s="8" t="n">
-        <v>6643</v>
+        <v>6205.04</v>
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
@@ -37978,11 +37976,11 @@
         </is>
       </c>
       <c r="F32" s="7" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>FL</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="H32" s="7" t="inlineStr">
@@ -37997,15 +37995,17 @@
       </c>
       <c r="J32" s="7" t="inlineStr">
         <is>
-          <t>01/16/2026</t>
+          <t>03/09/2026</t>
         </is>
       </c>
       <c r="K32" s="7" t="inlineStr">
         <is>
-          <t>01/12/2026</t>
-        </is>
-      </c>
-      <c r="L32" s="7" t="inlineStr"/>
+          <t>03/09/2026</t>
+        </is>
+      </c>
+      <c r="L32" s="7" t="n">
+        <v>3780576</v>
+      </c>
       <c r="M32" s="7" t="inlineStr">
         <is>
           <t>none</t>
@@ -38015,12 +38015,12 @@
     <row r="33">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>264034845083</t>
+          <t>264818442627</t>
         </is>
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>ARUMA TRANSPORT LLC</t>
+          <t>BOUNDLESS LOGISTICS LLC</t>
         </is>
       </c>
       <c r="C33" s="9" t="inlineStr">
@@ -38029,7 +38029,7 @@
         </is>
       </c>
       <c r="D33" s="10" t="n">
-        <v>6205.04</v>
+        <v>4174.4</v>
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
@@ -38037,7 +38037,7 @@
         </is>
       </c>
       <c r="F33" s="9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G33" s="9" t="inlineStr">
         <is>
@@ -38056,16 +38056,16 @@
       </c>
       <c r="J33" s="9" t="inlineStr">
         <is>
-          <t>03/09/2026</t>
+          <t>02/15/2026</t>
         </is>
       </c>
       <c r="K33" s="9" t="inlineStr">
         <is>
-          <t>03/09/2026</t>
+          <t>02/12/2026</t>
         </is>
       </c>
       <c r="L33" s="9" t="n">
-        <v>3780576</v>
+        <v>3924835</v>
       </c>
       <c r="M33" s="9" t="inlineStr">
         <is>
@@ -38076,12 +38076,12 @@
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>264818442627</t>
+          <t>269545282186</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>BOUNDLESS LOGISTICS LLC</t>
+          <t>J1S OPERATIONS LLC</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
@@ -38090,7 +38090,7 @@
         </is>
       </c>
       <c r="D34" s="8" t="n">
-        <v>4174.4</v>
+        <v>3796</v>
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
@@ -38102,68 +38102,64 @@
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>NC</t>
         </is>
       </c>
       <c r="H34" s="7" t="inlineStr">
         <is>
-          <t>AMC Agents LLC</t>
+          <t>American Fleet Insurance</t>
         </is>
       </c>
       <c r="I34" s="7" t="inlineStr">
         <is>
-          <t>Andres Piedrahita</t>
+          <t>Justin Feaster</t>
         </is>
       </c>
       <c r="J34" s="7" t="inlineStr">
         <is>
-          <t>02/15/2026</t>
+          <t>01/02/2026</t>
         </is>
       </c>
       <c r="K34" s="7" t="inlineStr">
         <is>
-          <t>02/12/2026</t>
+          <t>01/01/2026</t>
         </is>
       </c>
       <c r="L34" s="7" t="n">
-        <v>3924835</v>
+        <v>4336895</v>
       </c>
       <c r="M34" s="7" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>eld_only</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="9" t="inlineStr">
         <is>
-          <t>269545282186</t>
+          <t>265167986120</t>
         </is>
       </c>
       <c r="B35" s="9" t="inlineStr">
         <is>
-          <t>J1S OPERATIONS LLC</t>
+          <t>Timofey Shcherbina</t>
         </is>
       </c>
       <c r="C35" s="9" t="inlineStr">
         <is>
-          <t>Submitted</t>
+          <t>Waiting</t>
         </is>
       </c>
       <c r="D35" s="10" t="n">
-        <v>3796</v>
-      </c>
-      <c r="E35" s="9" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="E35" s="9" t="inlineStr"/>
       <c r="F35" s="9" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="G35" s="9" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="H35" s="9" t="inlineStr">
@@ -38178,32 +38174,26 @@
       </c>
       <c r="J35" s="9" t="inlineStr">
         <is>
-          <t>01/02/2026</t>
+          <t>01/06/2026</t>
         </is>
       </c>
       <c r="K35" s="9" t="inlineStr">
         <is>
-          <t>01/01/2026</t>
-        </is>
-      </c>
-      <c r="L35" s="9" t="n">
-        <v>4336895</v>
-      </c>
-      <c r="M35" s="9" t="inlineStr">
-        <is>
-          <t>eld_only</t>
-        </is>
-      </c>
+          <t>01/06/2026</t>
+        </is>
+      </c>
+      <c r="L35" s="9" t="inlineStr"/>
+      <c r="M35" s="9" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>265167986120</t>
+          <t>268639618524</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>Timofey Shcherbina</t>
+          <t>SUPER FREIGHT TRUCKING LLC</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
@@ -38216,11 +38206,11 @@
       </c>
       <c r="E36" s="7" t="inlineStr"/>
       <c r="F36" s="7" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>WA</t>
         </is>
       </c>
       <c r="H36" s="7" t="inlineStr">
@@ -38243,18 +38233,20 @@
           <t>01/06/2026</t>
         </is>
       </c>
-      <c r="L36" s="7" t="inlineStr"/>
+      <c r="L36" s="7" t="n">
+        <v>2455404</v>
+      </c>
       <c r="M36" s="7" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>268639618524</t>
+          <t>264513592821</t>
         </is>
       </c>
       <c r="B37" s="9" t="inlineStr">
         <is>
-          <t>SUPER FREIGHT TRUCKING LLC</t>
+          <t>DOMINIC'S TRANSPORT SERVICES LLC</t>
         </is>
       </c>
       <c r="C37" s="9" t="inlineStr">
@@ -38271,7 +38263,7 @@
       </c>
       <c r="G37" s="9" t="inlineStr">
         <is>
-          <t>WA</t>
+          <t>NC</t>
         </is>
       </c>
       <c r="H37" s="9" t="inlineStr">
@@ -38286,28 +38278,28 @@
       </c>
       <c r="J37" s="9" t="inlineStr">
         <is>
-          <t>01/06/2026</t>
+          <t>01/14/2026</t>
         </is>
       </c>
       <c r="K37" s="9" t="inlineStr">
         <is>
-          <t>01/06/2026</t>
+          <t>01/13/2026</t>
         </is>
       </c>
       <c r="L37" s="9" t="n">
-        <v>2455404</v>
+        <v>3410394</v>
       </c>
       <c r="M37" s="9" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>264513592821</t>
+          <t>261694648935</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>DOMINIC'S TRANSPORT SERVICES LLC</t>
+          <t>ALIF EXPRESS INC</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
@@ -38320,42 +38312,42 @@
       </c>
       <c r="E38" s="7" t="inlineStr"/>
       <c r="F38" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="H38" s="7" t="inlineStr">
         <is>
-          <t>American Fleet Insurance</t>
+          <t>Lone Star Direct Insurance Agency LLC</t>
         </is>
       </c>
       <c r="I38" s="7" t="inlineStr">
         <is>
-          <t>Justin Feaster</t>
+          <t>Zafarjon Khonkeldiev</t>
         </is>
       </c>
       <c r="J38" s="7" t="inlineStr">
         <is>
-          <t>01/14/2026</t>
+          <t>01/21/2026</t>
         </is>
       </c>
       <c r="K38" s="7" t="inlineStr">
         <is>
-          <t>01/13/2026</t>
+          <t>01/20/2026</t>
         </is>
       </c>
       <c r="L38" s="7" t="n">
-        <v>3410394</v>
+        <v>4176995</v>
       </c>
       <c r="M38" s="7" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="9" t="inlineStr">
         <is>
-          <t>261694648935</t>
+          <t>262838569886</t>
         </is>
       </c>
       <c r="B39" s="9" t="inlineStr">
@@ -38408,12 +38400,12 @@
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>262838569886</t>
+          <t>267435083285</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>ALIF EXPRESS INC</t>
+          <t>TRIPLE ACE HOTSHOT HAULING COMPANY LLC</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
@@ -38426,21 +38418,21 @@
       </c>
       <c r="E40" s="7" t="inlineStr"/>
       <c r="F40" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="H40" s="7" t="inlineStr">
         <is>
-          <t>Lone Star Direct Insurance Agency LLC</t>
+          <t>Insurance Leader Group, Inc</t>
         </is>
       </c>
       <c r="I40" s="7" t="inlineStr">
         <is>
-          <t>Zafarjon Khonkeldiev</t>
+          <t>Ivanoi Soto</t>
         </is>
       </c>
       <c r="J40" s="7" t="inlineStr">
@@ -38450,23 +38442,27 @@
       </c>
       <c r="K40" s="7" t="inlineStr">
         <is>
-          <t>01/20/2026</t>
+          <t>01/16/2026</t>
         </is>
       </c>
       <c r="L40" s="7" t="n">
-        <v>4176995</v>
-      </c>
-      <c r="M40" s="7" t="inlineStr"/>
+        <v>4448230</v>
+      </c>
+      <c r="M40" s="7" t="inlineStr">
+        <is>
+          <t>eld_only</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>267435083285</t>
+          <t>268777441285</t>
         </is>
       </c>
       <c r="B41" s="9" t="inlineStr">
         <is>
-          <t>TRIPLE ACE HOTSHOT HAULING COMPANY LLC</t>
+          <t>ADRIANO EXPRESS INC</t>
         </is>
       </c>
       <c r="C41" s="9" t="inlineStr">
@@ -38479,35 +38475,35 @@
       </c>
       <c r="E41" s="9" t="inlineStr"/>
       <c r="F41" s="9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G41" s="9" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>MI</t>
         </is>
       </c>
       <c r="H41" s="9" t="inlineStr">
         <is>
-          <t>Insurance Leader Group, Inc</t>
+          <t>American Fleet Insurance</t>
         </is>
       </c>
       <c r="I41" s="9" t="inlineStr">
         <is>
-          <t>Ivanoi Soto</t>
+          <t>Justin Feaster</t>
         </is>
       </c>
       <c r="J41" s="9" t="inlineStr">
         <is>
-          <t>01/21/2026</t>
+          <t>02/14/2026</t>
         </is>
       </c>
       <c r="K41" s="9" t="inlineStr">
         <is>
-          <t>01/16/2026</t>
+          <t>01/20/2026</t>
         </is>
       </c>
       <c r="L41" s="9" t="n">
-        <v>4448230</v>
+        <v>2317020</v>
       </c>
       <c r="M41" s="9" t="inlineStr">
         <is>
@@ -38518,12 +38514,12 @@
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>268777441285</t>
+          <t>262293586609</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>ADRIANO EXPRESS INC</t>
+          <t>A-MG TRUCKING LLC</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
@@ -38536,35 +38532,35 @@
       </c>
       <c r="E42" s="7" t="inlineStr"/>
       <c r="F42" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>MI</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="H42" s="7" t="inlineStr">
         <is>
-          <t>American Fleet Insurance</t>
+          <t>Insurance Leader Group, Inc</t>
         </is>
       </c>
       <c r="I42" s="7" t="inlineStr">
         <is>
-          <t>Justin Feaster</t>
+          <t>Ivanoi Soto</t>
         </is>
       </c>
       <c r="J42" s="7" t="inlineStr">
         <is>
-          <t>02/14/2026</t>
+          <t>04/10/2026</t>
         </is>
       </c>
       <c r="K42" s="7" t="inlineStr">
         <is>
-          <t>01/20/2026</t>
+          <t>01/22/2026</t>
         </is>
       </c>
       <c r="L42" s="7" t="n">
-        <v>2317020</v>
+        <v>4344886</v>
       </c>
       <c r="M42" s="7" t="inlineStr">
         <is>
@@ -38575,12 +38571,12 @@
     <row r="43">
       <c r="A43" s="9" t="inlineStr">
         <is>
-          <t>262293586609</t>
+          <t>262382436935</t>
         </is>
       </c>
       <c r="B43" s="9" t="inlineStr">
         <is>
-          <t>A-MG TRUCKING LLC</t>
+          <t>CKM AND KGR TRANSPORT LLC</t>
         </is>
       </c>
       <c r="C43" s="9" t="inlineStr">
@@ -38593,7 +38589,7 @@
       </c>
       <c r="E43" s="9" t="inlineStr"/>
       <c r="F43" s="9" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="G43" s="9" t="inlineStr">
         <is>
@@ -38602,26 +38598,26 @@
       </c>
       <c r="H43" s="9" t="inlineStr">
         <is>
-          <t>Insurance Leader Group, Inc</t>
+          <t>Connect Insurance Agency, Inc.</t>
         </is>
       </c>
       <c r="I43" s="9" t="inlineStr">
         <is>
-          <t>Ivanoi Soto</t>
+          <t>Jeremy Huddleston</t>
         </is>
       </c>
       <c r="J43" s="9" t="inlineStr">
         <is>
-          <t>04/10/2026</t>
+          <t>02/13/2026</t>
         </is>
       </c>
       <c r="K43" s="9" t="inlineStr">
         <is>
-          <t>01/22/2026</t>
+          <t>01/28/2026</t>
         </is>
       </c>
       <c r="L43" s="9" t="n">
-        <v>4344886</v>
+        <v>3192945</v>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
@@ -38632,12 +38628,12 @@
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>262382436935</t>
+          <t>266993641052</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>CKM AND KGR TRANSPORT LLC</t>
+          <t>RICH ROAD INC</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
@@ -38650,35 +38646,35 @@
       </c>
       <c r="E44" s="7" t="inlineStr"/>
       <c r="F44" s="7" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="H44" s="7" t="inlineStr">
         <is>
-          <t>Connect Insurance Agency, Inc.</t>
+          <t>Protectgo Services LLC</t>
         </is>
       </c>
       <c r="I44" s="7" t="inlineStr">
         <is>
-          <t>Jeremy Huddleston</t>
+          <t>Christopher Salazar</t>
         </is>
       </c>
       <c r="J44" s="7" t="inlineStr">
         <is>
-          <t>02/13/2026</t>
+          <t>01/30/2026</t>
         </is>
       </c>
       <c r="K44" s="7" t="inlineStr">
         <is>
-          <t>01/28/2026</t>
+          <t>01/26/2026</t>
         </is>
       </c>
       <c r="L44" s="7" t="n">
-        <v>3192945</v>
+        <v>4513800</v>
       </c>
       <c r="M44" s="7" t="inlineStr">
         <is>
@@ -38689,12 +38685,12 @@
     <row r="45">
       <c r="A45" s="9" t="inlineStr">
         <is>
-          <t>266993641052</t>
+          <t>261352984335</t>
         </is>
       </c>
       <c r="B45" s="9" t="inlineStr">
         <is>
-          <t>RICH ROAD INC</t>
+          <t>COASTAL SERVICE EXPRESS INC</t>
         </is>
       </c>
       <c r="C45" s="9" t="inlineStr">
@@ -38707,35 +38703,35 @@
       </c>
       <c r="E45" s="9" t="inlineStr"/>
       <c r="F45" s="9" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G45" s="9" t="inlineStr">
         <is>
-          <t>FL</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="H45" s="9" t="inlineStr">
         <is>
-          <t>Protectgo Services LLC</t>
+          <t>American Fleet Insurance</t>
         </is>
       </c>
       <c r="I45" s="9" t="inlineStr">
         <is>
-          <t>Christopher Salazar</t>
+          <t>Justin Feaster</t>
         </is>
       </c>
       <c r="J45" s="9" t="inlineStr">
         <is>
-          <t>01/30/2026</t>
+          <t>03/01/2026</t>
         </is>
       </c>
       <c r="K45" s="9" t="inlineStr">
         <is>
-          <t>01/26/2026</t>
+          <t>02/04/2026</t>
         </is>
       </c>
       <c r="L45" s="9" t="n">
-        <v>4513800</v>
+        <v>97819</v>
       </c>
       <c r="M45" s="9" t="inlineStr">
         <is>
@@ -38746,12 +38742,12 @@
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>261352984335</t>
+          <t>265202574010</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>COASTAL SERVICE EXPRESS INC</t>
+          <t>SIX GIRLS ONE BOY TRUCKING INC</t>
         </is>
       </c>
       <c r="C46" s="7" t="inlineStr">
@@ -38764,35 +38760,35 @@
       </c>
       <c r="E46" s="7" t="inlineStr"/>
       <c r="F46" s="7" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="H46" s="7" t="inlineStr">
         <is>
-          <t>American Fleet Insurance</t>
+          <t>AMC Agents LLC</t>
         </is>
       </c>
       <c r="I46" s="7" t="inlineStr">
         <is>
-          <t>Justin Feaster</t>
+          <t>Andres Piedrahita</t>
         </is>
       </c>
       <c r="J46" s="7" t="inlineStr">
         <is>
-          <t>03/01/2026</t>
+          <t>02/18/2026</t>
         </is>
       </c>
       <c r="K46" s="7" t="inlineStr">
         <is>
-          <t>02/04/2026</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="L46" s="7" t="n">
-        <v>97819</v>
+        <v>2112795</v>
       </c>
       <c r="M46" s="7" t="inlineStr">
         <is>
@@ -38803,12 +38799,12 @@
     <row r="47">
       <c r="A47" s="9" t="inlineStr">
         <is>
-          <t>265202574010</t>
+          <t>266713031267</t>
         </is>
       </c>
       <c r="B47" s="9" t="inlineStr">
         <is>
-          <t>SIX GIRLS ONE BOY TRUCKING INC</t>
+          <t>KUMAR TRANSPORT LLC</t>
         </is>
       </c>
       <c r="C47" s="9" t="inlineStr">
@@ -38821,11 +38817,11 @@
       </c>
       <c r="E47" s="9" t="inlineStr"/>
       <c r="F47" s="9" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G47" s="9" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="H47" s="9" t="inlineStr">
@@ -38835,21 +38831,21 @@
       </c>
       <c r="I47" s="9" t="inlineStr">
         <is>
-          <t>Andres Piedrahita</t>
+          <t>Carlos Ochoa</t>
         </is>
       </c>
       <c r="J47" s="9" t="inlineStr">
         <is>
-          <t>02/18/2026</t>
+          <t>02/14/2026</t>
         </is>
       </c>
       <c r="K47" s="9" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>02/06/2026</t>
         </is>
       </c>
       <c r="L47" s="9" t="n">
-        <v>2112795</v>
+        <v>4016247</v>
       </c>
       <c r="M47" s="9" t="inlineStr">
         <is>
@@ -38860,12 +38856,12 @@
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>266713031267</t>
+          <t>263780930303</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>KUMAR TRANSPORT LLC</t>
+          <t>CARLOS GONZALES</t>
         </is>
       </c>
       <c r="C48" s="7" t="inlineStr">
@@ -38878,7 +38874,7 @@
       </c>
       <c r="E48" s="7" t="inlineStr"/>
       <c r="F48" s="7" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
@@ -38887,12 +38883,12 @@
       </c>
       <c r="H48" s="7" t="inlineStr">
         <is>
-          <t>AMC Agents LLC</t>
+          <t>Tremach Inc</t>
         </is>
       </c>
       <c r="I48" s="7" t="inlineStr">
         <is>
-          <t>Carlos Ochoa</t>
+          <t>Angie Del Toro</t>
         </is>
       </c>
       <c r="J48" s="7" t="inlineStr">
@@ -38902,11 +38898,11 @@
       </c>
       <c r="K48" s="7" t="inlineStr">
         <is>
-          <t>02/06/2026</t>
+          <t>02/13/2026</t>
         </is>
       </c>
       <c r="L48" s="7" t="n">
-        <v>4016247</v>
+        <v>632179</v>
       </c>
       <c r="M48" s="7" t="inlineStr">
         <is>
@@ -38917,12 +38913,12 @@
     <row r="49">
       <c r="A49" s="9" t="inlineStr">
         <is>
-          <t>263780930303</t>
+          <t>260743900895</t>
         </is>
       </c>
       <c r="B49" s="9" t="inlineStr">
         <is>
-          <t>CARLOS GONZALES</t>
+          <t>TERRAZAS TRANSPORTATION LLC</t>
         </is>
       </c>
       <c r="C49" s="9" t="inlineStr">
@@ -38935,7 +38931,7 @@
       </c>
       <c r="E49" s="9" t="inlineStr"/>
       <c r="F49" s="9" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="G49" s="9" t="inlineStr">
         <is>
@@ -38944,26 +38940,26 @@
       </c>
       <c r="H49" s="9" t="inlineStr">
         <is>
-          <t>Tremach Inc</t>
+          <t>AGENTRUBEN.COM LLC</t>
         </is>
       </c>
       <c r="I49" s="9" t="inlineStr">
         <is>
-          <t>Angie Del Toro</t>
+          <t>RUBEN Saucedo</t>
         </is>
       </c>
       <c r="J49" s="9" t="inlineStr">
         <is>
-          <t>02/14/2026</t>
+          <t>02/21/2026</t>
         </is>
       </c>
       <c r="K49" s="9" t="inlineStr">
         <is>
-          <t>02/13/2026</t>
+          <t>02/20/2026</t>
         </is>
       </c>
       <c r="L49" s="9" t="n">
-        <v>632179</v>
+        <v>2991712</v>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
@@ -38974,12 +38970,12 @@
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>260743900895</t>
+          <t>261503419029</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>TERRAZAS TRANSPORTATION LLC</t>
+          <t>RIKI LOGISTICS LLC</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr">
@@ -38992,7 +38988,7 @@
       </c>
       <c r="E50" s="7" t="inlineStr"/>
       <c r="F50" s="7" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="G50" s="7" t="inlineStr">
         <is>
@@ -39001,42 +38997,38 @@
       </c>
       <c r="H50" s="7" t="inlineStr">
         <is>
-          <t>AGENTRUBEN.COM LLC</t>
+          <t>AMC Agents LLC</t>
         </is>
       </c>
       <c r="I50" s="7" t="inlineStr">
         <is>
-          <t>RUBEN Saucedo</t>
+          <t>Andres Piedrahita</t>
         </is>
       </c>
       <c r="J50" s="7" t="inlineStr">
         <is>
-          <t>02/21/2026</t>
+          <t>02/28/2026</t>
         </is>
       </c>
       <c r="K50" s="7" t="inlineStr">
         <is>
-          <t>02/20/2026</t>
+          <t>02/27/2026</t>
         </is>
       </c>
       <c r="L50" s="7" t="n">
-        <v>2991712</v>
-      </c>
-      <c r="M50" s="7" t="inlineStr">
-        <is>
-          <t>eld_only</t>
-        </is>
-      </c>
+        <v>4178122</v>
+      </c>
+      <c r="M50" s="7" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="9" t="inlineStr">
         <is>
-          <t>261503419029</t>
+          <t>264074990034</t>
         </is>
       </c>
       <c r="B51" s="9" t="inlineStr">
         <is>
-          <t>RIKI LOGISTICS LLC</t>
+          <t>MANNY EXPRESS LLC</t>
         </is>
       </c>
       <c r="C51" s="9" t="inlineStr">
@@ -39049,11 +39041,11 @@
       </c>
       <c r="E51" s="9" t="inlineStr"/>
       <c r="F51" s="9" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G51" s="9" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="H51" s="9" t="inlineStr">
@@ -39063,33 +39055,37 @@
       </c>
       <c r="I51" s="9" t="inlineStr">
         <is>
-          <t>Andres Piedrahita</t>
+          <t>Carlos Ochoa</t>
         </is>
       </c>
       <c r="J51" s="9" t="inlineStr">
         <is>
-          <t>02/28/2026</t>
+          <t>02/26/2026</t>
         </is>
       </c>
       <c r="K51" s="9" t="inlineStr">
         <is>
-          <t>02/27/2026</t>
+          <t>02/24/2026</t>
         </is>
       </c>
       <c r="L51" s="9" t="n">
-        <v>4178122</v>
-      </c>
-      <c r="M51" s="9" t="inlineStr"/>
+        <v>4189204</v>
+      </c>
+      <c r="M51" s="9" t="inlineStr">
+        <is>
+          <t>eld_only</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>264074990034</t>
+          <t>268040248090</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>MANNY EXPRESS LLC</t>
+          <t>GLOBAL STAR ENTERPRISES INC</t>
         </is>
       </c>
       <c r="C52" s="7" t="inlineStr">
@@ -39102,35 +39098,35 @@
       </c>
       <c r="E52" s="7" t="inlineStr"/>
       <c r="F52" s="7" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G52" s="7" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="H52" s="7" t="inlineStr">
         <is>
-          <t>AMC Agents LLC</t>
+          <t>InsurNorth Corp</t>
         </is>
       </c>
       <c r="I52" s="7" t="inlineStr">
         <is>
-          <t>Carlos Ochoa</t>
+          <t>Mark Fabyanchuk</t>
         </is>
       </c>
       <c r="J52" s="7" t="inlineStr">
         <is>
+          <t>02/27/2026</t>
+        </is>
+      </c>
+      <c r="K52" s="7" t="inlineStr">
+        <is>
           <t>02/26/2026</t>
         </is>
       </c>
-      <c r="K52" s="7" t="inlineStr">
-        <is>
-          <t>02/24/2026</t>
-        </is>
-      </c>
       <c r="L52" s="7" t="n">
-        <v>4189204</v>
+        <v>4264731</v>
       </c>
       <c r="M52" s="7" t="inlineStr">
         <is>
@@ -39141,12 +39137,12 @@
     <row r="53">
       <c r="A53" s="9" t="inlineStr">
         <is>
-          <t>268040248090</t>
+          <t>268303729063</t>
         </is>
       </c>
       <c r="B53" s="9" t="inlineStr">
         <is>
-          <t>GLOBAL STAR ENTERPRISES INC</t>
+          <t>ROBERTOM TRANSPORTATION LLC</t>
         </is>
       </c>
       <c r="C53" s="9" t="inlineStr">
@@ -39159,35 +39155,35 @@
       </c>
       <c r="E53" s="9" t="inlineStr"/>
       <c r="F53" s="9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G53" s="9" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="H53" s="9" t="inlineStr">
         <is>
-          <t>InsurNorth Corp</t>
+          <t>AMC Agents LLC</t>
         </is>
       </c>
       <c r="I53" s="9" t="inlineStr">
         <is>
-          <t>Mark Fabyanchuk</t>
+          <t>Andres Piedrahita</t>
         </is>
       </c>
       <c r="J53" s="9" t="inlineStr">
         <is>
-          <t>02/27/2026</t>
+          <t>02/26/2026</t>
         </is>
       </c>
       <c r="K53" s="9" t="inlineStr">
         <is>
-          <t>02/26/2026</t>
+          <t>02/25/2026</t>
         </is>
       </c>
       <c r="L53" s="9" t="n">
-        <v>4264731</v>
+        <v>2914305</v>
       </c>
       <c r="M53" s="9" t="inlineStr">
         <is>
@@ -39198,12 +39194,12 @@
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>268303729063</t>
+          <t>260292846354</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>ROBERTOM TRANSPORTATION LLC</t>
+          <t>ONTIMECHASE INC</t>
         </is>
       </c>
       <c r="C54" s="7" t="inlineStr">
@@ -39216,51 +39212,47 @@
       </c>
       <c r="E54" s="7" t="inlineStr"/>
       <c r="F54" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G54" s="7" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="H54" s="7" t="inlineStr">
         <is>
-          <t>AMC Agents LLC</t>
+          <t>Lone Star Direct Insurance Agency LLC</t>
         </is>
       </c>
       <c r="I54" s="7" t="inlineStr">
         <is>
-          <t>Andres Piedrahita</t>
+          <t>Zafarjon Khonkeldiev</t>
         </is>
       </c>
       <c r="J54" s="7" t="inlineStr">
         <is>
-          <t>02/26/2026</t>
+          <t>03/28/2026</t>
         </is>
       </c>
       <c r="K54" s="7" t="inlineStr">
         <is>
-          <t>02/25/2026</t>
+          <t>03/27/2026</t>
         </is>
       </c>
       <c r="L54" s="7" t="n">
-        <v>2914305</v>
-      </c>
-      <c r="M54" s="7" t="inlineStr">
-        <is>
-          <t>eld_only</t>
-        </is>
-      </c>
+        <v>3957346</v>
+      </c>
+      <c r="M54" s="7" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="9" t="inlineStr">
         <is>
-          <t>260292846354</t>
+          <t>260549364550</t>
         </is>
       </c>
       <c r="B55" s="9" t="inlineStr">
         <is>
-          <t>ONTIMECHASE INC</t>
+          <t>DANIEL TRUCKING PRO INC</t>
         </is>
       </c>
       <c r="C55" s="9" t="inlineStr">
@@ -39273,47 +39265,51 @@
       </c>
       <c r="E55" s="9" t="inlineStr"/>
       <c r="F55" s="9" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G55" s="9" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="H55" s="9" t="inlineStr">
         <is>
-          <t>Lone Star Direct Insurance Agency LLC</t>
+          <t>American Fleet Insurance</t>
         </is>
       </c>
       <c r="I55" s="9" t="inlineStr">
         <is>
-          <t>Zafarjon Khonkeldiev</t>
+          <t>Justin Feaster</t>
         </is>
       </c>
       <c r="J55" s="9" t="inlineStr">
         <is>
-          <t>03/28/2026</t>
+          <t>03/21/2026</t>
         </is>
       </c>
       <c r="K55" s="9" t="inlineStr">
         <is>
-          <t>03/27/2026</t>
+          <t>03/20/2026</t>
         </is>
       </c>
       <c r="L55" s="9" t="n">
-        <v>3957346</v>
-      </c>
-      <c r="M55" s="9" t="inlineStr"/>
+        <v>3584147</v>
+      </c>
+      <c r="M55" s="9" t="inlineStr">
+        <is>
+          <t>eld_only</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>260549364550</t>
+          <t>260573647554</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>DANIEL TRUCKING PRO INC</t>
+          <t>CAESAR TRANSPORT LLC</t>
         </is>
       </c>
       <c r="C56" s="7" t="inlineStr">
@@ -39330,31 +39326,31 @@
       </c>
       <c r="G56" s="7" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>UT</t>
         </is>
       </c>
       <c r="H56" s="7" t="inlineStr">
         <is>
-          <t>American Fleet Insurance</t>
+          <t>Protectgo Services LLC</t>
         </is>
       </c>
       <c r="I56" s="7" t="inlineStr">
         <is>
-          <t>Justin Feaster</t>
+          <t>Christopher Salazar</t>
         </is>
       </c>
       <c r="J56" s="7" t="inlineStr">
         <is>
-          <t>03/21/2026</t>
+          <t>04/22/2026</t>
         </is>
       </c>
       <c r="K56" s="7" t="inlineStr">
         <is>
-          <t>03/20/2026</t>
+          <t>03/27/2026</t>
         </is>
       </c>
       <c r="L56" s="7" t="n">
-        <v>3584147</v>
+        <v>2347760</v>
       </c>
       <c r="M56" s="7" t="inlineStr">
         <is>
@@ -39365,12 +39361,12 @@
     <row r="57">
       <c r="A57" s="9" t="inlineStr">
         <is>
-          <t>260573647554</t>
+          <t>261350139916</t>
         </is>
       </c>
       <c r="B57" s="9" t="inlineStr">
         <is>
-          <t>CAESAR TRANSPORT LLC</t>
+          <t>ONTIMECHASE INC</t>
         </is>
       </c>
       <c r="C57" s="9" t="inlineStr">
@@ -39383,51 +39379,47 @@
       </c>
       <c r="E57" s="9" t="inlineStr"/>
       <c r="F57" s="9" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G57" s="9" t="inlineStr">
         <is>
-          <t>UT</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="H57" s="9" t="inlineStr">
         <is>
-          <t>Protectgo Services LLC</t>
+          <t>Lone Star Direct Insurance Agency LLC</t>
         </is>
       </c>
       <c r="I57" s="9" t="inlineStr">
         <is>
-          <t>Christopher Salazar</t>
+          <t>Zafarjon Khonkeldiev</t>
         </is>
       </c>
       <c r="J57" s="9" t="inlineStr">
         <is>
-          <t>04/22/2026</t>
+          <t>03/27/2026</t>
         </is>
       </c>
       <c r="K57" s="9" t="inlineStr">
         <is>
-          <t>03/27/2026</t>
+          <t>03/26/2026</t>
         </is>
       </c>
       <c r="L57" s="9" t="n">
-        <v>2347760</v>
-      </c>
-      <c r="M57" s="9" t="inlineStr">
-        <is>
-          <t>eld_only</t>
-        </is>
-      </c>
+        <v>3957346</v>
+      </c>
+      <c r="M57" s="9" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
         <is>
-          <t>261350139916</t>
+          <t>262083542111</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>ONTIMECHASE INC</t>
+          <t>FACUNDO MENDEZ REYES</t>
         </is>
       </c>
       <c r="C58" s="7" t="inlineStr">
@@ -39440,47 +39432,47 @@
       </c>
       <c r="E58" s="7" t="inlineStr"/>
       <c r="F58" s="7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G58" s="7" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="H58" s="7" t="inlineStr">
         <is>
-          <t>Lone Star Direct Insurance Agency LLC</t>
+          <t>Protectgo Services LLC</t>
         </is>
       </c>
       <c r="I58" s="7" t="inlineStr">
         <is>
-          <t>Zafarjon Khonkeldiev</t>
+          <t>Christopher Salazar</t>
         </is>
       </c>
       <c r="J58" s="7" t="inlineStr">
         <is>
-          <t>03/27/2026</t>
+          <t>03/23/2026</t>
         </is>
       </c>
       <c r="K58" s="7" t="inlineStr">
         <is>
-          <t>03/26/2026</t>
+          <t>03/22/2026</t>
         </is>
       </c>
       <c r="L58" s="7" t="n">
-        <v>3957346</v>
+        <v>3187408</v>
       </c>
       <c r="M58" s="7" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="9" t="inlineStr">
         <is>
-          <t>262083542111</t>
+          <t>262520794648</t>
         </is>
       </c>
       <c r="B59" s="9" t="inlineStr">
         <is>
-          <t>FACUNDO MENDEZ REYES</t>
+          <t>NATIONWIDE HAULING INC</t>
         </is>
       </c>
       <c r="C59" s="9" t="inlineStr">
@@ -39497,43 +39489,43 @@
       </c>
       <c r="G59" s="9" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>OR</t>
         </is>
       </c>
       <c r="H59" s="9" t="inlineStr">
         <is>
-          <t>Protectgo Services LLC</t>
+          <t>Resolute Insurance Group LLC</t>
         </is>
       </c>
       <c r="I59" s="9" t="inlineStr">
         <is>
-          <t>Christopher Salazar</t>
+          <t>Josh Connor</t>
         </is>
       </c>
       <c r="J59" s="9" t="inlineStr">
         <is>
-          <t>03/23/2026</t>
+          <t>03/05/2026</t>
         </is>
       </c>
       <c r="K59" s="9" t="inlineStr">
         <is>
-          <t>03/22/2026</t>
+          <t>03/04/2026</t>
         </is>
       </c>
       <c r="L59" s="9" t="n">
-        <v>3187408</v>
+        <v>2097487</v>
       </c>
       <c r="M59" s="9" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
         <is>
-          <t>262520794648</t>
+          <t>262620542162</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>NATIONWIDE HAULING INC</t>
+          <t>ONTIMECHASE INC</t>
         </is>
       </c>
       <c r="C60" s="7" t="inlineStr">
@@ -39546,42 +39538,42 @@
       </c>
       <c r="E60" s="7" t="inlineStr"/>
       <c r="F60" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G60" s="7" t="inlineStr">
         <is>
-          <t>OR</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="H60" s="7" t="inlineStr">
         <is>
-          <t>Resolute Insurance Group LLC</t>
+          <t>Lone Star Direct Insurance Agency LLC</t>
         </is>
       </c>
       <c r="I60" s="7" t="inlineStr">
         <is>
-          <t>Josh Connor</t>
+          <t>Zafarjon Khonkeldiev</t>
         </is>
       </c>
       <c r="J60" s="7" t="inlineStr">
         <is>
-          <t>03/05/2026</t>
+          <t>03/28/2026</t>
         </is>
       </c>
       <c r="K60" s="7" t="inlineStr">
         <is>
-          <t>03/04/2026</t>
+          <t>03/27/2026</t>
         </is>
       </c>
       <c r="L60" s="7" t="n">
-        <v>2097487</v>
+        <v>3957346</v>
       </c>
       <c r="M60" s="7" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="9" t="inlineStr">
         <is>
-          <t>262620542162</t>
+          <t>262621161792</t>
         </is>
       </c>
       <c r="B61" s="9" t="inlineStr">
@@ -39599,7 +39591,7 @@
       </c>
       <c r="E61" s="9" t="inlineStr"/>
       <c r="F61" s="9" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="G61" s="9" t="inlineStr">
         <is>
@@ -39608,38 +39600,42 @@
       </c>
       <c r="H61" s="9" t="inlineStr">
         <is>
-          <t>Lone Star Direct Insurance Agency LLC</t>
+          <t>InsurNorth Corp</t>
         </is>
       </c>
       <c r="I61" s="9" t="inlineStr">
         <is>
-          <t>Zafarjon Khonkeldiev</t>
+          <t>Ali Boyko</t>
         </is>
       </c>
       <c r="J61" s="9" t="inlineStr">
         <is>
-          <t>03/28/2026</t>
+          <t>03/31/2026</t>
         </is>
       </c>
       <c r="K61" s="9" t="inlineStr">
         <is>
-          <t>03/27/2026</t>
+          <t>03/30/2026</t>
         </is>
       </c>
       <c r="L61" s="9" t="n">
         <v>3957346</v>
       </c>
-      <c r="M61" s="9" t="inlineStr"/>
+      <c r="M61" s="9" t="inlineStr">
+        <is>
+          <t>eld_only</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
         <is>
-          <t>262621161792</t>
+          <t>262735300483</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
         <is>
-          <t>ONTIMECHASE INC</t>
+          <t>ACHINT TRUCKING INC</t>
         </is>
       </c>
       <c r="C62" s="7" t="inlineStr">
@@ -39652,35 +39648,35 @@
       </c>
       <c r="E62" s="7" t="inlineStr"/>
       <c r="F62" s="7" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="G62" s="7" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="H62" s="7" t="inlineStr">
         <is>
-          <t>InsurNorth Corp</t>
+          <t>Connect Insurance Agency, Inc.</t>
         </is>
       </c>
       <c r="I62" s="7" t="inlineStr">
         <is>
-          <t>Ali Boyko</t>
+          <t>Jeremy Huddleston</t>
         </is>
       </c>
       <c r="J62" s="7" t="inlineStr">
         <is>
-          <t>03/31/2026</t>
+          <t>03/24/2026</t>
         </is>
       </c>
       <c r="K62" s="7" t="inlineStr">
         <is>
-          <t>03/30/2026</t>
+          <t>03/23/2026</t>
         </is>
       </c>
       <c r="L62" s="7" t="n">
-        <v>3957346</v>
+        <v>2056659</v>
       </c>
       <c r="M62" s="7" t="inlineStr">
         <is>
@@ -39691,12 +39687,12 @@
     <row r="63">
       <c r="A63" s="9" t="inlineStr">
         <is>
-          <t>262735300483</t>
+          <t>262842967180</t>
         </is>
       </c>
       <c r="B63" s="9" t="inlineStr">
         <is>
-          <t>ACHINT TRUCKING INC</t>
+          <t>ADY TRANSPORT LLC</t>
         </is>
       </c>
       <c r="C63" s="9" t="inlineStr">
@@ -39709,35 +39705,35 @@
       </c>
       <c r="E63" s="9" t="inlineStr"/>
       <c r="F63" s="9" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="G63" s="9" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="H63" s="9" t="inlineStr">
         <is>
-          <t>Connect Insurance Agency, Inc.</t>
+          <t>Resolute Insurance Group LLC</t>
         </is>
       </c>
       <c r="I63" s="9" t="inlineStr">
         <is>
-          <t>Jeremy Huddleston</t>
+          <t>Josh Connor</t>
         </is>
       </c>
       <c r="J63" s="9" t="inlineStr">
         <is>
-          <t>03/24/2026</t>
+          <t>03/15/2026</t>
         </is>
       </c>
       <c r="K63" s="9" t="inlineStr">
         <is>
-          <t>03/23/2026</t>
+          <t>03/05/2026</t>
         </is>
       </c>
       <c r="L63" s="9" t="n">
-        <v>2056659</v>
+        <v>3594665</v>
       </c>
       <c r="M63" s="9" t="inlineStr">
         <is>
@@ -39748,12 +39744,12 @@
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
         <is>
-          <t>262842967180</t>
+          <t>264544915404</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
         <is>
-          <t>ADY TRANSPORT LLC</t>
+          <t>VELOCITY CARGO INC</t>
         </is>
       </c>
       <c r="C64" s="7" t="inlineStr">
@@ -39766,35 +39762,35 @@
       </c>
       <c r="E64" s="7" t="inlineStr"/>
       <c r="F64" s="7" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="G64" s="7" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="H64" s="7" t="inlineStr">
         <is>
-          <t>Resolute Insurance Group LLC</t>
+          <t>Dream Assurance LLC</t>
         </is>
       </c>
       <c r="I64" s="7" t="inlineStr">
         <is>
-          <t>Josh Connor</t>
+          <t>Kevin Patrick Morrissy</t>
         </is>
       </c>
       <c r="J64" s="7" t="inlineStr">
         <is>
-          <t>03/15/2026</t>
+          <t>03/17/2026</t>
         </is>
       </c>
       <c r="K64" s="7" t="inlineStr">
         <is>
-          <t>03/05/2026</t>
+          <t>03/16/2026</t>
         </is>
       </c>
       <c r="L64" s="7" t="n">
-        <v>3594665</v>
+        <v>4202687</v>
       </c>
       <c r="M64" s="7" t="inlineStr">
         <is>
@@ -39805,12 +39801,12 @@
     <row r="65">
       <c r="A65" s="9" t="inlineStr">
         <is>
-          <t>264544915404</t>
+          <t>264923752419</t>
         </is>
       </c>
       <c r="B65" s="9" t="inlineStr">
         <is>
-          <t>VELOCITY CARGO INC</t>
+          <t>UR4 TRANSPORTATION LLC</t>
         </is>
       </c>
       <c r="C65" s="9" t="inlineStr">
@@ -39823,94 +39819,37 @@
       </c>
       <c r="E65" s="9" t="inlineStr"/>
       <c r="F65" s="9" t="n">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="G65" s="9" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="H65" s="9" t="inlineStr">
         <is>
-          <t>Dream Assurance LLC</t>
+          <t>American Fleet Insurance</t>
         </is>
       </c>
       <c r="I65" s="9" t="inlineStr">
         <is>
-          <t>Kevin Patrick Morrissy</t>
+          <t>Justin Feaster</t>
         </is>
       </c>
       <c r="J65" s="9" t="inlineStr">
         <is>
+          <t>03/18/2026</t>
+        </is>
+      </c>
+      <c r="K65" s="9" t="inlineStr">
+        <is>
           <t>03/17/2026</t>
         </is>
       </c>
-      <c r="K65" s="9" t="inlineStr">
-        <is>
-          <t>03/16/2026</t>
-        </is>
-      </c>
       <c r="L65" s="9" t="n">
-        <v>4202687</v>
+        <v>4264094</v>
       </c>
       <c r="M65" s="9" t="inlineStr">
-        <is>
-          <t>eld_only</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="7" t="inlineStr">
-        <is>
-          <t>264923752419</t>
-        </is>
-      </c>
-      <c r="B66" s="7" t="inlineStr">
-        <is>
-          <t>UR4 TRANSPORTATION LLC</t>
-        </is>
-      </c>
-      <c r="C66" s="7" t="inlineStr">
-        <is>
-          <t>Waiting</t>
-        </is>
-      </c>
-      <c r="D66" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E66" s="7" t="inlineStr"/>
-      <c r="F66" s="7" t="n">
-        <v>24</v>
-      </c>
-      <c r="G66" s="7" t="inlineStr">
-        <is>
-          <t>IL</t>
-        </is>
-      </c>
-      <c r="H66" s="7" t="inlineStr">
-        <is>
-          <t>American Fleet Insurance</t>
-        </is>
-      </c>
-      <c r="I66" s="7" t="inlineStr">
-        <is>
-          <t>Justin Feaster</t>
-        </is>
-      </c>
-      <c r="J66" s="7" t="inlineStr">
-        <is>
-          <t>03/18/2026</t>
-        </is>
-      </c>
-      <c r="K66" s="7" t="inlineStr">
-        <is>
-          <t>03/17/2026</t>
-        </is>
-      </c>
-      <c r="L66" s="7" t="n">
-        <v>4264094</v>
-      </c>
-      <c r="M66" s="7" t="inlineStr">
         <is>
           <t>eld_only</t>
         </is>

</xml_diff>

<commit_message>
Daily rebuild Sat 05/30/2026  7:59:29.99
</commit_message>
<xml_diff>
--- a/generated/Fleet Pipeline/BDM_Fleet_Pipeline_Report.xlsx
+++ b/generated/Fleet Pipeline/BDM_Fleet_Pipeline_Report.xlsx
@@ -494,10 +494,10 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C2" s="4" t="n">
-        <v>2188089.6</v>
+        <v>2101692.16</v>
       </c>
     </row>
     <row r="3">
@@ -536,7 +536,7 @@
         <v>187</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>10317084.14</v>
+        <v>10288777.99</v>
       </c>
     </row>
     <row r="6">
@@ -17748,7 +17748,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M35"/>
+  <dimension ref="A1:M34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -17958,29 +17958,29 @@
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>263881557291</t>
+          <t>260280669582</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>LALA TRUCKLINE INC</t>
+          <t>NORTH STATES LOGISTICS</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>Quoted</t>
+          <t>Submitted</t>
         </is>
       </c>
       <c r="D4" s="8" t="n">
-        <v>86397.44</v>
+        <v>393845.35</v>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F4" s="7" t="n">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
@@ -17989,26 +17989,26 @@
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>Amerigo Insurance Agency</t>
+          <t>Aic Insurance Agency LLC</t>
         </is>
       </c>
       <c r="I4" s="7" t="inlineStr">
         <is>
-          <t>Parmjit Dhami</t>
+          <t>Tanya Golovina</t>
         </is>
       </c>
       <c r="J4" s="7" t="inlineStr">
         <is>
-          <t>05/22/2026</t>
+          <t>02/26/2026</t>
         </is>
       </c>
       <c r="K4" s="7" t="inlineStr">
         <is>
-          <t>02/22/2026</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="L4" s="7" t="n">
-        <v>4036826</v>
+        <v>3155337</v>
       </c>
       <c r="M4" s="7" t="inlineStr">
         <is>
@@ -18019,12 +18019,12 @@
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>260280669582</t>
+          <t>260927812922</t>
         </is>
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>NORTH STATES LOGISTICS</t>
+          <t>FORCE TRANS INC</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
@@ -18033,7 +18033,7 @@
         </is>
       </c>
       <c r="D5" s="10" t="n">
-        <v>393845.35</v>
+        <v>369286.73</v>
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
@@ -18041,7 +18041,7 @@
         </is>
       </c>
       <c r="F5" s="9" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
@@ -18050,26 +18050,26 @@
       </c>
       <c r="H5" s="9" t="inlineStr">
         <is>
-          <t>Aic Insurance Agency LLC</t>
+          <t>Insurance Mobile Services, Inc.</t>
         </is>
       </c>
       <c r="I5" s="9" t="inlineStr">
         <is>
-          <t>Tanya Golovina</t>
+          <t>Paul Metlenko</t>
         </is>
       </c>
       <c r="J5" s="9" t="inlineStr">
         <is>
-          <t>02/26/2026</t>
+          <t>01/09/2026</t>
         </is>
       </c>
       <c r="K5" s="9" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>01/09/2026</t>
         </is>
       </c>
       <c r="L5" s="9" t="n">
-        <v>3155337</v>
+        <v>2327228</v>
       </c>
       <c r="M5" s="9" t="inlineStr">
         <is>
@@ -18080,12 +18080,12 @@
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>260927812922</t>
+          <t>262132006063</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>FORCE TRANS INC</t>
+          <t>SHAH TRUCKLINE INC</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
@@ -18094,7 +18094,7 @@
         </is>
       </c>
       <c r="D6" s="8" t="n">
-        <v>369286.73</v>
+        <v>359368.51</v>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
@@ -18102,7 +18102,7 @@
         </is>
       </c>
       <c r="F6" s="7" t="n">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
@@ -18111,26 +18111,26 @@
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>Insurance Mobile Services, Inc.</t>
+          <t>Network Truck Insurance Services, Inc.</t>
         </is>
       </c>
       <c r="I6" s="7" t="inlineStr">
         <is>
-          <t>Paul Metlenko</t>
+          <t>Carey Avitua</t>
         </is>
       </c>
       <c r="J6" s="7" t="inlineStr">
         <is>
-          <t>01/09/2026</t>
+          <t>03/13/2026</t>
         </is>
       </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>01/09/2026</t>
+          <t>03/09/2026</t>
         </is>
       </c>
       <c r="L6" s="7" t="n">
-        <v>2327228</v>
+        <v>2776606</v>
       </c>
       <c r="M6" s="7" t="inlineStr">
         <is>
@@ -18141,12 +18141,12 @@
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>262132006063</t>
+          <t>262055717127</t>
         </is>
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>SHAH TRUCKLINE INC</t>
+          <t>MUSHIANA EXPRESS LLC</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
@@ -18155,7 +18155,7 @@
         </is>
       </c>
       <c r="D7" s="10" t="n">
-        <v>359368.51</v>
+        <v>158992.07</v>
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
@@ -18163,35 +18163,35 @@
         </is>
       </c>
       <c r="F7" s="9" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>UT</t>
         </is>
       </c>
       <c r="H7" s="9" t="inlineStr">
         <is>
-          <t>Network Truck Insurance Services, Inc.</t>
+          <t>Amerigo Insurance Agency</t>
         </is>
       </c>
       <c r="I7" s="9" t="inlineStr">
         <is>
-          <t>Carey Avitua</t>
+          <t>Parmjit Dhami</t>
         </is>
       </c>
       <c r="J7" s="9" t="inlineStr">
         <is>
-          <t>03/13/2026</t>
+          <t>04/20/2026</t>
         </is>
       </c>
       <c r="K7" s="9" t="inlineStr">
         <is>
-          <t>03/09/2026</t>
+          <t>01/21/2026</t>
         </is>
       </c>
       <c r="L7" s="9" t="n">
-        <v>2776606</v>
+        <v>1934301</v>
       </c>
       <c r="M7" s="9" t="inlineStr">
         <is>
@@ -18202,12 +18202,12 @@
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>262055717127</t>
+          <t>268608695265</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>MUSHIANA EXPRESS LLC</t>
+          <t>BEST FREIGHTLINES INC</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
@@ -18216,7 +18216,7 @@
         </is>
       </c>
       <c r="D8" s="8" t="n">
-        <v>158992.07</v>
+        <v>106060.57</v>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
@@ -18224,35 +18224,35 @@
         </is>
       </c>
       <c r="F8" s="7" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>UT</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>Amerigo Insurance Agency</t>
+          <t>Stellar Management, Inc</t>
         </is>
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
-          <t>Parmjit Dhami</t>
+          <t>Raman Palta</t>
         </is>
       </c>
       <c r="J8" s="7" t="inlineStr">
         <is>
-          <t>04/20/2026</t>
+          <t>02/01/2026</t>
         </is>
       </c>
       <c r="K8" s="7" t="inlineStr">
         <is>
-          <t>01/21/2026</t>
+          <t>01/26/2026</t>
         </is>
       </c>
       <c r="L8" s="7" t="n">
-        <v>1934301</v>
+        <v>1312590</v>
       </c>
       <c r="M8" s="7" t="inlineStr">
         <is>
@@ -18263,12 +18263,12 @@
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>268608695265</t>
+          <t>262460684935</t>
         </is>
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>BEST FREIGHTLINES INC</t>
+          <t>P G TRANS INC</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
@@ -18277,59 +18277,59 @@
         </is>
       </c>
       <c r="D9" s="10" t="n">
-        <v>106060.57</v>
+        <v>11773.74</v>
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F9" s="9" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="H9" s="9" t="inlineStr">
         <is>
-          <t>Stellar Management, Inc</t>
+          <t>American Continental Insurance Services Inc</t>
         </is>
       </c>
       <c r="I9" s="9" t="inlineStr">
         <is>
-          <t>Raman Palta</t>
+          <t>Raman Kailey</t>
         </is>
       </c>
       <c r="J9" s="9" t="inlineStr">
         <is>
-          <t>02/01/2026</t>
+          <t>01/17/2026</t>
         </is>
       </c>
       <c r="K9" s="9" t="inlineStr">
         <is>
-          <t>01/26/2026</t>
+          <t>01/15/2026</t>
         </is>
       </c>
       <c r="L9" s="9" t="n">
-        <v>1312590</v>
+        <v>2329219</v>
       </c>
       <c r="M9" s="9" t="inlineStr">
         <is>
-          <t>eld_only</t>
+          <t>none</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>262460684935</t>
+          <t>266528160888</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>P G TRANS INC</t>
+          <t>VVV LOGISTICS INC</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
@@ -18338,7 +18338,7 @@
         </is>
       </c>
       <c r="D10" s="8" t="n">
-        <v>11773.74</v>
+        <v>8563.200000000001</v>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
@@ -18346,51 +18346,51 @@
         </is>
       </c>
       <c r="F10" s="7" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>NC</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>American Continental Insurance Services Inc</t>
+          <t>Aic Insurance Agency LLC</t>
         </is>
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>Raman Kailey</t>
+          <t>Grigoriy Gasan</t>
         </is>
       </c>
       <c r="J10" s="7" t="inlineStr">
         <is>
-          <t>01/17/2026</t>
+          <t>01/31/2026</t>
         </is>
       </c>
       <c r="K10" s="7" t="inlineStr">
         <is>
-          <t>01/15/2026</t>
+          <t>01/08/2026</t>
         </is>
       </c>
       <c r="L10" s="7" t="n">
-        <v>2329219</v>
+        <v>2330993</v>
       </c>
       <c r="M10" s="7" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>eld_only</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>266528160888</t>
+          <t>262967085690</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>VVV LOGISTICS INC</t>
+          <t>KAVKAZ WAY LLC</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
@@ -18399,7 +18399,7 @@
         </is>
       </c>
       <c r="D11" s="10" t="n">
-        <v>8563.200000000001</v>
+        <v>8107.05</v>
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
@@ -18407,11 +18407,11 @@
         </is>
       </c>
       <c r="F11" s="9" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="H11" s="9" t="inlineStr">
@@ -18421,37 +18421,37 @@
       </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t>Grigoriy Gasan</t>
+          <t>Dmitri Omelco</t>
         </is>
       </c>
       <c r="J11" s="9" t="inlineStr">
         <is>
-          <t>01/31/2026</t>
+          <t>03/21/2026</t>
         </is>
       </c>
       <c r="K11" s="9" t="inlineStr">
         <is>
-          <t>01/08/2026</t>
+          <t>03/13/2026</t>
         </is>
       </c>
       <c r="L11" s="9" t="n">
-        <v>2330993</v>
+        <v>4214405</v>
       </c>
       <c r="M11" s="9" t="inlineStr">
         <is>
-          <t>eld_only</t>
+          <t>none</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>262967085690</t>
+          <t>261701906587</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>KAVKAZ WAY LLC</t>
+          <t>GN TRUCKLINES INC</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
@@ -18460,7 +18460,7 @@
         </is>
       </c>
       <c r="D12" s="8" t="n">
-        <v>8107.05</v>
+        <v>6643</v>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
@@ -18468,35 +18468,35 @@
         </is>
       </c>
       <c r="F12" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>Aic Insurance Agency LLC</t>
+          <t>Stellar Management, Inc</t>
         </is>
       </c>
       <c r="I12" s="7" t="inlineStr">
         <is>
-          <t>Dmitri Omelco</t>
+          <t>Raman Palta</t>
         </is>
       </c>
       <c r="J12" s="7" t="inlineStr">
         <is>
-          <t>03/21/2026</t>
+          <t>03/06/2026</t>
         </is>
       </c>
       <c r="K12" s="7" t="inlineStr">
         <is>
-          <t>03/13/2026</t>
+          <t>02/09/2026</t>
         </is>
       </c>
       <c r="L12" s="7" t="n">
-        <v>4214405</v>
+        <v>3772590</v>
       </c>
       <c r="M12" s="7" t="inlineStr">
         <is>
@@ -18507,12 +18507,12 @@
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
         <is>
-          <t>261701906587</t>
+          <t>266006213124</t>
         </is>
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>GN TRUCKLINES INC</t>
+          <t>SUNSTAR TRANSPORT INC</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
@@ -18521,7 +18521,7 @@
         </is>
       </c>
       <c r="D13" s="10" t="n">
-        <v>6643</v>
+        <v>6619.02</v>
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
@@ -18529,7 +18529,7 @@
         </is>
       </c>
       <c r="F13" s="9" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
@@ -18538,26 +18538,26 @@
       </c>
       <c r="H13" s="9" t="inlineStr">
         <is>
-          <t>Stellar Management, Inc</t>
+          <t>Alex Rue Insurance Agency, Inc</t>
         </is>
       </c>
       <c r="I13" s="9" t="inlineStr">
         <is>
-          <t>Raman Palta</t>
+          <t>Alexander Rue</t>
         </is>
       </c>
       <c r="J13" s="9" t="inlineStr">
         <is>
-          <t>03/06/2026</t>
+          <t>03/15/2026</t>
         </is>
       </c>
       <c r="K13" s="9" t="inlineStr">
         <is>
-          <t>02/09/2026</t>
+          <t>02/12/2026</t>
         </is>
       </c>
       <c r="L13" s="9" t="n">
-        <v>3772590</v>
+        <v>2880906</v>
       </c>
       <c r="M13" s="9" t="inlineStr">
         <is>
@@ -18568,12 +18568,12 @@
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>266006213124</t>
+          <t>268660737784</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>SUNSTAR TRANSPORT INC</t>
+          <t>HILLS FREIGHT LLC</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
@@ -18582,43 +18582,39 @@
         </is>
       </c>
       <c r="D14" s="8" t="n">
-        <v>6619.02</v>
-      </c>
-      <c r="E14" s="7" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="E14" s="7" t="inlineStr"/>
       <c r="F14" s="7" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>NV</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>Alex Rue Insurance Agency, Inc</t>
+          <t>Insurance Mobile Services, Inc.</t>
         </is>
       </c>
       <c r="I14" s="7" t="inlineStr">
         <is>
-          <t>Alexander Rue</t>
+          <t>Paul Metlenko</t>
         </is>
       </c>
       <c r="J14" s="7" t="inlineStr">
         <is>
-          <t>03/15/2026</t>
+          <t>03/05/2026</t>
         </is>
       </c>
       <c r="K14" s="7" t="inlineStr">
         <is>
-          <t>02/12/2026</t>
+          <t>02/18/2026</t>
         </is>
       </c>
       <c r="L14" s="7" t="n">
-        <v>2880906</v>
+        <v>853290</v>
       </c>
       <c r="M14" s="7" t="inlineStr">
         <is>
@@ -18629,17 +18625,17 @@
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>268660737784</t>
+          <t>265534014081</t>
         </is>
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>HILLS FREIGHT LLC</t>
+          <t>BLAZE TRANSPORT LLC</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>Submitted</t>
+          <t>Waiting</t>
         </is>
       </c>
       <c r="D15" s="10" t="n">
@@ -18647,51 +18643,47 @@
       </c>
       <c r="E15" s="9" t="inlineStr"/>
       <c r="F15" s="9" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="G15" s="9" t="inlineStr">
         <is>
-          <t>NV</t>
+          <t>VA</t>
         </is>
       </c>
       <c r="H15" s="9" t="inlineStr">
         <is>
-          <t>Insurance Mobile Services, Inc.</t>
+          <t>American Continental Insurance Services Inc</t>
         </is>
       </c>
       <c r="I15" s="9" t="inlineStr">
         <is>
-          <t>Paul Metlenko</t>
+          <t>Raman Kailey</t>
         </is>
       </c>
       <c r="J15" s="9" t="inlineStr">
         <is>
-          <t>03/05/2026</t>
+          <t>01/06/2026</t>
         </is>
       </c>
       <c r="K15" s="9" t="inlineStr">
         <is>
-          <t>02/18/2026</t>
+          <t>01/05/2026</t>
         </is>
       </c>
       <c r="L15" s="9" t="n">
-        <v>853290</v>
-      </c>
-      <c r="M15" s="9" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
+        <v>4224716</v>
+      </c>
+      <c r="M15" s="9" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>265534014081</t>
+          <t>269375817975</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>BLAZE TRANSPORT LLC</t>
+          <t>B NICE TRANSPORT INC</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
@@ -18708,22 +18700,22 @@
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>VA</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>American Continental Insurance Services Inc</t>
+          <t>A.S.I.A Inc</t>
         </is>
       </c>
       <c r="I16" s="7" t="inlineStr">
         <is>
-          <t>Raman Kailey</t>
+          <t>Deepak Goswami</t>
         </is>
       </c>
       <c r="J16" s="7" t="inlineStr">
         <is>
-          <t>01/06/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="K16" s="7" t="inlineStr">
@@ -18732,19 +18724,23 @@
         </is>
       </c>
       <c r="L16" s="7" t="n">
-        <v>4224716</v>
-      </c>
-      <c r="M16" s="7" t="inlineStr"/>
+        <v>4073911</v>
+      </c>
+      <c r="M16" s="7" t="inlineStr">
+        <is>
+          <t>eld_only</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>269375817975</t>
+          <t>261412929134</t>
         </is>
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>B NICE TRANSPORT INC</t>
+          <t>BIRRING TRUCKING INC</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
@@ -18757,35 +18753,35 @@
       </c>
       <c r="E17" s="9" t="inlineStr"/>
       <c r="F17" s="9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G17" s="9" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="H17" s="9" t="inlineStr">
         <is>
-          <t>A.S.I.A Inc</t>
+          <t>Amerigo Insurance Agency</t>
         </is>
       </c>
       <c r="I17" s="9" t="inlineStr">
         <is>
-          <t>Deepak Goswami</t>
+          <t>Parmjit Dhami</t>
         </is>
       </c>
       <c r="J17" s="9" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>01/31/2026</t>
         </is>
       </c>
       <c r="K17" s="9" t="inlineStr">
         <is>
-          <t>01/05/2026</t>
+          <t>01/20/2026</t>
         </is>
       </c>
       <c r="L17" s="9" t="n">
-        <v>4073911</v>
+        <v>2337721</v>
       </c>
       <c r="M17" s="9" t="inlineStr">
         <is>
@@ -18796,12 +18792,12 @@
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>261412929134</t>
+          <t>266354483626</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>BIRRING TRUCKING INC</t>
+          <t>ROBUST LLC</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
@@ -18814,35 +18810,35 @@
       </c>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="H18" s="7" t="inlineStr">
         <is>
-          <t>Amerigo Insurance Agency</t>
+          <t>A.S.I.A Inc</t>
         </is>
       </c>
       <c r="I18" s="7" t="inlineStr">
         <is>
-          <t>Parmjit Dhami</t>
+          <t>Deepak Goswami</t>
         </is>
       </c>
       <c r="J18" s="7" t="inlineStr">
         <is>
-          <t>01/31/2026</t>
+          <t>01/17/2026</t>
         </is>
       </c>
       <c r="K18" s="7" t="inlineStr">
         <is>
-          <t>01/20/2026</t>
+          <t>01/16/2026</t>
         </is>
       </c>
       <c r="L18" s="7" t="n">
-        <v>2337721</v>
+        <v>4230983</v>
       </c>
       <c r="M18" s="7" t="inlineStr">
         <is>
@@ -18853,12 +18849,12 @@
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>266354483626</t>
+          <t>269953313884</t>
         </is>
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>ROBUST LLC</t>
+          <t>PATWAL TRANS INC</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
@@ -18875,31 +18871,31 @@
       </c>
       <c r="G19" s="9" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="H19" s="9" t="inlineStr">
         <is>
-          <t>A.S.I.A Inc</t>
+          <t>Stellar Management, Inc</t>
         </is>
       </c>
       <c r="I19" s="9" t="inlineStr">
         <is>
-          <t>Deepak Goswami</t>
+          <t>Raman Palta</t>
         </is>
       </c>
       <c r="J19" s="9" t="inlineStr">
         <is>
-          <t>01/17/2026</t>
+          <t>02/17/2026</t>
         </is>
       </c>
       <c r="K19" s="9" t="inlineStr">
         <is>
-          <t>01/16/2026</t>
+          <t>01/21/2026</t>
         </is>
       </c>
       <c r="L19" s="9" t="n">
-        <v>4230983</v>
+        <v>3386779</v>
       </c>
       <c r="M19" s="9" t="inlineStr">
         <is>
@@ -18910,12 +18906,12 @@
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>269953313884</t>
+          <t>262522868735</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>PATWAL TRANS INC</t>
+          <t>CVB TRANSPORTATION LLC</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
@@ -18937,26 +18933,26 @@
       </c>
       <c r="H20" s="7" t="inlineStr">
         <is>
-          <t>Stellar Management, Inc</t>
+          <t>Network Truck Insurance Services, Inc.</t>
         </is>
       </c>
       <c r="I20" s="7" t="inlineStr">
         <is>
-          <t>Raman Palta</t>
+          <t>Ben Hanson</t>
         </is>
       </c>
       <c r="J20" s="7" t="inlineStr">
         <is>
-          <t>02/17/2026</t>
+          <t>02/02/2026</t>
         </is>
       </c>
       <c r="K20" s="7" t="inlineStr">
         <is>
-          <t>01/21/2026</t>
+          <t>01/29/2026</t>
         </is>
       </c>
       <c r="L20" s="7" t="n">
-        <v>3386779</v>
+        <v>4022321</v>
       </c>
       <c r="M20" s="7" t="inlineStr">
         <is>
@@ -18967,12 +18963,12 @@
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>262522868735</t>
+          <t>265580560499</t>
         </is>
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>CVB TRANSPORTATION LLC</t>
+          <t>FORCE TRANS INC</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
@@ -18985,7 +18981,7 @@
       </c>
       <c r="E21" s="9" t="inlineStr"/>
       <c r="F21" s="9" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="G21" s="9" t="inlineStr">
         <is>
@@ -18994,17 +18990,17 @@
       </c>
       <c r="H21" s="9" t="inlineStr">
         <is>
-          <t>Network Truck Insurance Services, Inc.</t>
+          <t>Insurance Mobile Services, Inc.</t>
         </is>
       </c>
       <c r="I21" s="9" t="inlineStr">
         <is>
-          <t>Ben Hanson</t>
+          <t>Paul Metlenko</t>
         </is>
       </c>
       <c r="J21" s="9" t="inlineStr">
         <is>
-          <t>02/02/2026</t>
+          <t>02/01/2026</t>
         </is>
       </c>
       <c r="K21" s="9" t="inlineStr">
@@ -19013,23 +19009,23 @@
         </is>
       </c>
       <c r="L21" s="9" t="n">
-        <v>4022321</v>
+        <v>2327228</v>
       </c>
       <c r="M21" s="9" t="inlineStr">
         <is>
-          <t>eld_only</t>
+          <t>none</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>265580560499</t>
+          <t>263542064667</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>FORCE TRANS INC</t>
+          <t>ALL ROUTES TRUCKING INC</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
@@ -19042,51 +19038,47 @@
       </c>
       <c r="E22" s="7" t="inlineStr"/>
       <c r="F22" s="7" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>CT</t>
         </is>
       </c>
       <c r="H22" s="7" t="inlineStr">
         <is>
-          <t>Insurance Mobile Services, Inc.</t>
+          <t>A.S.I.A Inc</t>
         </is>
       </c>
       <c r="I22" s="7" t="inlineStr">
         <is>
-          <t>Paul Metlenko</t>
+          <t>Shubham Kamra</t>
         </is>
       </c>
       <c r="J22" s="7" t="inlineStr">
         <is>
-          <t>02/01/2026</t>
+          <t>02/04/2026</t>
         </is>
       </c>
       <c r="K22" s="7" t="inlineStr">
         <is>
-          <t>01/29/2026</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="L22" s="7" t="n">
-        <v>2327228</v>
-      </c>
-      <c r="M22" s="7" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
+        <v>3773202</v>
+      </c>
+      <c r="M22" s="7" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>263542064667</t>
+          <t>267880450970</t>
         </is>
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>ALL ROUTES TRUCKING INC</t>
+          <t>SPS TRANS CARGO INC</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
@@ -19099,47 +19091,47 @@
       </c>
       <c r="E23" s="9" t="inlineStr"/>
       <c r="F23" s="9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G23" s="9" t="inlineStr">
         <is>
-          <t>CT</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="H23" s="9" t="inlineStr">
         <is>
-          <t>A.S.I.A Inc</t>
+          <t>Soho Insurance Brokerage, Inc.</t>
         </is>
       </c>
       <c r="I23" s="9" t="inlineStr">
         <is>
-          <t>Shubham Kamra</t>
+          <t>Parmpaul Thandi</t>
         </is>
       </c>
       <c r="J23" s="9" t="inlineStr">
         <is>
-          <t>02/04/2026</t>
+          <t>02/07/2026</t>
         </is>
       </c>
       <c r="K23" s="9" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>02/06/2026</t>
         </is>
       </c>
       <c r="L23" s="9" t="n">
-        <v>3773202</v>
+        <v>4150917</v>
       </c>
       <c r="M23" s="9" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>267880450970</t>
+          <t>269233409466</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>SPS TRANS CARGO INC</t>
+          <t>STONEFIRE TRANSPORT INC</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
@@ -19152,7 +19144,7 @@
       </c>
       <c r="E24" s="7" t="inlineStr"/>
       <c r="F24" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
@@ -19161,38 +19153,38 @@
       </c>
       <c r="H24" s="7" t="inlineStr">
         <is>
-          <t>Soho Insurance Brokerage, Inc.</t>
+          <t>Amerigo Insurance Agency</t>
         </is>
       </c>
       <c r="I24" s="7" t="inlineStr">
         <is>
-          <t>Parmpaul Thandi</t>
+          <t>Parmjit Dhami</t>
         </is>
       </c>
       <c r="J24" s="7" t="inlineStr">
         <is>
-          <t>02/07/2026</t>
+          <t>02/14/2026</t>
         </is>
       </c>
       <c r="K24" s="7" t="inlineStr">
         <is>
-          <t>02/06/2026</t>
+          <t>02/14/2026</t>
         </is>
       </c>
       <c r="L24" s="7" t="n">
-        <v>4150917</v>
+        <v>4356732</v>
       </c>
       <c r="M24" s="7" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>269233409466</t>
+          <t>264975565305</t>
         </is>
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>STONEFIRE TRANSPORT INC</t>
+          <t>MAJHA TRANSPORTATION INC</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
@@ -19205,47 +19197,51 @@
       </c>
       <c r="E25" s="9" t="inlineStr"/>
       <c r="F25" s="9" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G25" s="9" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>VA</t>
         </is>
       </c>
       <c r="H25" s="9" t="inlineStr">
         <is>
-          <t>Amerigo Insurance Agency</t>
+          <t>MST INSURANCE SERVICES INC</t>
         </is>
       </c>
       <c r="I25" s="9" t="inlineStr">
         <is>
-          <t>Parmjit Dhami</t>
+          <t>Manmdeep Thiara</t>
         </is>
       </c>
       <c r="J25" s="9" t="inlineStr">
         <is>
-          <t>02/14/2026</t>
+          <t>02/20/2026</t>
         </is>
       </c>
       <c r="K25" s="9" t="inlineStr">
         <is>
-          <t>02/14/2026</t>
+          <t>02/16/2026</t>
         </is>
       </c>
       <c r="L25" s="9" t="n">
-        <v>4356732</v>
-      </c>
-      <c r="M25" s="9" t="inlineStr"/>
+        <v>3547788</v>
+      </c>
+      <c r="M25" s="9" t="inlineStr">
+        <is>
+          <t>eld_only</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>264975565305</t>
+          <t>267109923027</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>MAJHA TRANSPORTATION INC</t>
+          <t>SKYRIDE TRANSPORT INC</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
@@ -19258,51 +19254,47 @@
       </c>
       <c r="E26" s="7" t="inlineStr"/>
       <c r="F26" s="7" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>VA</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="H26" s="7" t="inlineStr">
         <is>
-          <t>MST INSURANCE SERVICES INC</t>
+          <t>A.S.I.A Inc</t>
         </is>
       </c>
       <c r="I26" s="7" t="inlineStr">
         <is>
-          <t>Manmdeep Thiara</t>
+          <t>Shubham Kamra</t>
         </is>
       </c>
       <c r="J26" s="7" t="inlineStr">
         <is>
-          <t>02/20/2026</t>
+          <t>02/25/2026</t>
         </is>
       </c>
       <c r="K26" s="7" t="inlineStr">
         <is>
-          <t>02/16/2026</t>
+          <t>02/24/2026</t>
         </is>
       </c>
       <c r="L26" s="7" t="n">
-        <v>3547788</v>
-      </c>
-      <c r="M26" s="7" t="inlineStr">
-        <is>
-          <t>eld_only</t>
-        </is>
-      </c>
+        <v>4359531</v>
+      </c>
+      <c r="M26" s="7" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>267109923027</t>
+          <t>260623480943</t>
         </is>
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>SKYRIDE TRANSPORT INC</t>
+          <t>OZZIE'S TRUCKING INC</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
@@ -19315,7 +19307,7 @@
       </c>
       <c r="E27" s="9" t="inlineStr"/>
       <c r="F27" s="9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G27" s="9" t="inlineStr">
         <is>
@@ -19324,38 +19316,42 @@
       </c>
       <c r="H27" s="9" t="inlineStr">
         <is>
-          <t>A.S.I.A Inc</t>
+          <t>Network Truck Insurance Services, Inc.</t>
         </is>
       </c>
       <c r="I27" s="9" t="inlineStr">
         <is>
-          <t>Shubham Kamra</t>
+          <t>Colby Novielli</t>
         </is>
       </c>
       <c r="J27" s="9" t="inlineStr">
         <is>
-          <t>02/25/2026</t>
+          <t>03/04/2026</t>
         </is>
       </c>
       <c r="K27" s="9" t="inlineStr">
         <is>
-          <t>02/24/2026</t>
+          <t>03/05/2026</t>
         </is>
       </c>
       <c r="L27" s="9" t="n">
-        <v>4359531</v>
-      </c>
-      <c r="M27" s="9" t="inlineStr"/>
+        <v>2931415</v>
+      </c>
+      <c r="M27" s="9" t="inlineStr">
+        <is>
+          <t>eld_only</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>260623480943</t>
+          <t>262778489832</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>OZZIE'S TRUCKING INC</t>
+          <t>PRESERVER TRANS LLC</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
@@ -19368,7 +19364,7 @@
       </c>
       <c r="E28" s="7" t="inlineStr"/>
       <c r="F28" s="7" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
@@ -19377,26 +19373,26 @@
       </c>
       <c r="H28" s="7" t="inlineStr">
         <is>
-          <t>Network Truck Insurance Services, Inc.</t>
+          <t>Alex Rue Insurance Agency, Inc</t>
         </is>
       </c>
       <c r="I28" s="7" t="inlineStr">
         <is>
-          <t>Colby Novielli</t>
+          <t>Alexander Rue</t>
         </is>
       </c>
       <c r="J28" s="7" t="inlineStr">
         <is>
-          <t>03/04/2026</t>
+          <t>03/17/2026</t>
         </is>
       </c>
       <c r="K28" s="7" t="inlineStr">
         <is>
-          <t>03/05/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="L28" s="7" t="n">
-        <v>2931415</v>
+        <v>2985316</v>
       </c>
       <c r="M28" s="7" t="inlineStr">
         <is>
@@ -19407,12 +19403,12 @@
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>262778489832</t>
+          <t>262824950523</t>
         </is>
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>PRESERVER TRANS LLC</t>
+          <t>S BHANGU LLC</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
@@ -19425,7 +19421,7 @@
       </c>
       <c r="E29" s="9" t="inlineStr"/>
       <c r="F29" s="9" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="G29" s="9" t="inlineStr">
         <is>
@@ -19434,12 +19430,12 @@
       </c>
       <c r="H29" s="9" t="inlineStr">
         <is>
-          <t>Alex Rue Insurance Agency, Inc</t>
+          <t>Monumental Insurance Services, LLC</t>
         </is>
       </c>
       <c r="I29" s="9" t="inlineStr">
         <is>
-          <t>Alexander Rue</t>
+          <t>Omar Morquecho</t>
         </is>
       </c>
       <c r="J29" s="9" t="inlineStr">
@@ -19449,11 +19445,11 @@
       </c>
       <c r="K29" s="9" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>03/16/2026</t>
         </is>
       </c>
       <c r="L29" s="9" t="n">
-        <v>2985316</v>
+        <v>3097539</v>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
@@ -19464,12 +19460,12 @@
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>262824950523</t>
+          <t>263725382869</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>S BHANGU LLC</t>
+          <t>PROGRESS TRUCKING INC</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
@@ -19482,7 +19478,7 @@
       </c>
       <c r="E30" s="7" t="inlineStr"/>
       <c r="F30" s="7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
@@ -19491,26 +19487,26 @@
       </c>
       <c r="H30" s="7" t="inlineStr">
         <is>
-          <t>Monumental Insurance Services, LLC</t>
+          <t>A.S.I.A Inc</t>
         </is>
       </c>
       <c r="I30" s="7" t="inlineStr">
         <is>
-          <t>Omar Morquecho</t>
+          <t>Deepak Goswami</t>
         </is>
       </c>
       <c r="J30" s="7" t="inlineStr">
         <is>
-          <t>03/17/2026</t>
+          <t>03/03/2026</t>
         </is>
       </c>
       <c r="K30" s="7" t="inlineStr">
         <is>
-          <t>03/16/2026</t>
+          <t>03/02/2026</t>
         </is>
       </c>
       <c r="L30" s="7" t="n">
-        <v>3097539</v>
+        <v>3093909</v>
       </c>
       <c r="M30" s="7" t="inlineStr">
         <is>
@@ -19521,12 +19517,12 @@
     <row r="31">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>263725382869</t>
+          <t>264014006562</t>
         </is>
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>PROGRESS TRUCKING INC</t>
+          <t>PANNU HOLDING CARRIER LLC</t>
         </is>
       </c>
       <c r="C31" s="9" t="inlineStr">
@@ -19543,22 +19539,22 @@
       </c>
       <c r="G31" s="9" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>WA</t>
         </is>
       </c>
       <c r="H31" s="9" t="inlineStr">
         <is>
-          <t>A.S.I.A Inc</t>
+          <t>Stellar Management, Inc</t>
         </is>
       </c>
       <c r="I31" s="9" t="inlineStr">
         <is>
-          <t>Deepak Goswami</t>
+          <t>Raman Palta</t>
         </is>
       </c>
       <c r="J31" s="9" t="inlineStr">
         <is>
-          <t>03/03/2026</t>
+          <t>04/10/2026</t>
         </is>
       </c>
       <c r="K31" s="9" t="inlineStr">
@@ -19567,7 +19563,7 @@
         </is>
       </c>
       <c r="L31" s="9" t="n">
-        <v>3093909</v>
+        <v>3428765</v>
       </c>
       <c r="M31" s="9" t="inlineStr">
         <is>
@@ -19578,12 +19574,12 @@
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>264014006562</t>
+          <t>264266931323</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>PANNU HOLDING CARRIER LLC</t>
+          <t>KC FREIGHT LLC</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
@@ -19596,35 +19592,35 @@
       </c>
       <c r="E32" s="7" t="inlineStr"/>
       <c r="F32" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>WA</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="H32" s="7" t="inlineStr">
         <is>
-          <t>Stellar Management, Inc</t>
+          <t>A.S.I.A Inc</t>
         </is>
       </c>
       <c r="I32" s="7" t="inlineStr">
         <is>
-          <t>Raman Palta</t>
+          <t>Shubham Kamra</t>
         </is>
       </c>
       <c r="J32" s="7" t="inlineStr">
         <is>
-          <t>04/10/2026</t>
+          <t>04/01/2026</t>
         </is>
       </c>
       <c r="K32" s="7" t="inlineStr">
         <is>
-          <t>03/02/2026</t>
+          <t>03/31/2026</t>
         </is>
       </c>
       <c r="L32" s="7" t="n">
-        <v>3428765</v>
+        <v>2631633</v>
       </c>
       <c r="M32" s="7" t="inlineStr">
         <is>
@@ -19635,12 +19631,12 @@
     <row r="33">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>264266931323</t>
+          <t>264689973799</t>
         </is>
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>KC FREIGHT LLC</t>
+          <t>ALPHA CARRIER LLC</t>
         </is>
       </c>
       <c r="C33" s="9" t="inlineStr">
@@ -19653,35 +19649,35 @@
       </c>
       <c r="E33" s="9" t="inlineStr"/>
       <c r="F33" s="9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G33" s="9" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="H33" s="9" t="inlineStr">
         <is>
-          <t>A.S.I.A Inc</t>
+          <t>Stellar Management, Inc</t>
         </is>
       </c>
       <c r="I33" s="9" t="inlineStr">
         <is>
-          <t>Shubham Kamra</t>
+          <t>Raman Palta</t>
         </is>
       </c>
       <c r="J33" s="9" t="inlineStr">
         <is>
-          <t>04/01/2026</t>
+          <t>05/05/2026</t>
         </is>
       </c>
       <c r="K33" s="9" t="inlineStr">
         <is>
-          <t>03/31/2026</t>
+          <t>03/02/2026</t>
         </is>
       </c>
       <c r="L33" s="9" t="n">
-        <v>2631633</v>
+        <v>4008627</v>
       </c>
       <c r="M33" s="9" t="inlineStr">
         <is>
@@ -19692,12 +19688,12 @@
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>264689973799</t>
+          <t>265331970134</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>ALPHA CARRIER LLC</t>
+          <t>S BHANGU LLC</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
@@ -19710,94 +19706,37 @@
       </c>
       <c r="E34" s="7" t="inlineStr"/>
       <c r="F34" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="H34" s="7" t="inlineStr">
         <is>
-          <t>Stellar Management, Inc</t>
+          <t>Monumental Insurance Services, LLC</t>
         </is>
       </c>
       <c r="I34" s="7" t="inlineStr">
         <is>
-          <t>Raman Palta</t>
+          <t>Omar Morquecho</t>
         </is>
       </c>
       <c r="J34" s="7" t="inlineStr">
         <is>
-          <t>05/05/2026</t>
+          <t>03/18/2026</t>
         </is>
       </c>
       <c r="K34" s="7" t="inlineStr">
         <is>
-          <t>03/02/2026</t>
+          <t>03/17/2026</t>
         </is>
       </c>
       <c r="L34" s="7" t="n">
-        <v>4008627</v>
+        <v>3097539</v>
       </c>
       <c r="M34" s="7" t="inlineStr">
-        <is>
-          <t>eld_only</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="9" t="inlineStr">
-        <is>
-          <t>265331970134</t>
-        </is>
-      </c>
-      <c r="B35" s="9" t="inlineStr">
-        <is>
-          <t>S BHANGU LLC</t>
-        </is>
-      </c>
-      <c r="C35" s="9" t="inlineStr">
-        <is>
-          <t>Waiting</t>
-        </is>
-      </c>
-      <c r="D35" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E35" s="9" t="inlineStr"/>
-      <c r="F35" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G35" s="9" t="inlineStr">
-        <is>
-          <t>CA</t>
-        </is>
-      </c>
-      <c r="H35" s="9" t="inlineStr">
-        <is>
-          <t>Monumental Insurance Services, LLC</t>
-        </is>
-      </c>
-      <c r="I35" s="9" t="inlineStr">
-        <is>
-          <t>Omar Morquecho</t>
-        </is>
-      </c>
-      <c r="J35" s="9" t="inlineStr">
-        <is>
-          <t>03/18/2026</t>
-        </is>
-      </c>
-      <c r="K35" s="9" t="inlineStr">
-        <is>
-          <t>03/17/2026</t>
-        </is>
-      </c>
-      <c r="L35" s="9" t="n">
-        <v>3097539</v>
-      </c>
-      <c r="M35" s="9" t="inlineStr">
         <is>
           <t>eld_only</t>
         </is>
@@ -24835,12 +24774,12 @@
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>263902898771</t>
+          <t>263542089381</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>W&amp;T LOGISTICS INC</t>
+          <t>ADV TRUCKING LLC</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
@@ -24849,7 +24788,7 @@
         </is>
       </c>
       <c r="D8" s="8" t="n">
-        <v>51607.5</v>
+        <v>72274.50999999999</v>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
@@ -24861,31 +24800,31 @@
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>NJ</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>Reliance Partners, LLC</t>
+          <t>Empire Company Insurance Services, Inc.</t>
         </is>
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
-          <t>API_USER API_USER</t>
+          <t>Jennifer Reimers</t>
         </is>
       </c>
       <c r="J8" s="7" t="inlineStr">
         <is>
-          <t>04/19/2026</t>
+          <t>06/03/2026</t>
         </is>
       </c>
       <c r="K8" s="7" t="inlineStr">
         <is>
-          <t>03/24/2026</t>
+          <t>03/06/2026</t>
         </is>
       </c>
       <c r="L8" s="7" t="n">
-        <v>4219023</v>
+        <v>2070108</v>
       </c>
       <c r="M8" s="7" t="inlineStr">
         <is>
@@ -24896,12 +24835,12 @@
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>264024928386</t>
+          <t>263902898771</t>
         </is>
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>ECW TRANSPORTATION INC</t>
+          <t>W&amp;T LOGISTICS INC</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
@@ -24910,19 +24849,19 @@
         </is>
       </c>
       <c r="D9" s="10" t="n">
-        <v>9295.030000000001</v>
+        <v>51607.5</v>
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F9" s="9" t="n">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="H9" s="9" t="inlineStr">
@@ -24937,16 +24876,16 @@
       </c>
       <c r="J9" s="9" t="inlineStr">
         <is>
-          <t>04/20/2026</t>
+          <t>04/19/2026</t>
         </is>
       </c>
       <c r="K9" s="9" t="inlineStr">
         <is>
-          <t>03/12/2026</t>
+          <t>03/24/2026</t>
         </is>
       </c>
       <c r="L9" s="9" t="n">
-        <v>3046384</v>
+        <v>4219023</v>
       </c>
       <c r="M9" s="9" t="inlineStr">
         <is>
@@ -24957,57 +24896,57 @@
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>252087228306</t>
+          <t>264024928386</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>BABALA TRUCKING LLC</t>
+          <t>ECW TRANSPORTATION INC</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Quote Docs in Progress</t>
+          <t>In Review</t>
         </is>
       </c>
       <c r="D10" s="8" t="n">
-        <v>49006.29</v>
+        <v>9295.030000000001</v>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F10" s="7" t="n">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>WA</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>United Advantage Insurance Services</t>
+          <t>Reliance Partners, LLC</t>
         </is>
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>Khalid Salama</t>
+          <t>API_USER API_USER</t>
         </is>
       </c>
       <c r="J10" s="7" t="inlineStr">
         <is>
-          <t>11/14/2025</t>
+          <t>04/20/2026</t>
         </is>
       </c>
       <c r="K10" s="7" t="inlineStr">
         <is>
-          <t>02/09/2026</t>
+          <t>03/12/2026</t>
         </is>
       </c>
       <c r="L10" s="7" t="n">
-        <v>4224158</v>
+        <v>3046384</v>
       </c>
       <c r="M10" s="7" t="inlineStr">
         <is>
@@ -25018,57 +24957,57 @@
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>253174349440</t>
+          <t>252087228306</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>HANDSOME TRANSPORTATION INC</t>
+          <t>BABALA TRUCKING LLC</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>Quoted</t>
+          <t>Quote Docs in Progress</t>
         </is>
       </c>
       <c r="D11" s="10" t="n">
-        <v>548010.52</v>
+        <v>49006.29</v>
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F11" s="9" t="n">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>WA</t>
         </is>
       </c>
       <c r="H11" s="9" t="inlineStr">
         <is>
-          <t>Safeline Insurance Agency, Inc.</t>
+          <t>United Advantage Insurance Services</t>
         </is>
       </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t>Gohar Aramyan</t>
+          <t>Khalid Salama</t>
         </is>
       </c>
       <c r="J11" s="9" t="inlineStr">
         <is>
-          <t>08/18/2025</t>
+          <t>11/14/2025</t>
         </is>
       </c>
       <c r="K11" s="9" t="inlineStr">
         <is>
-          <t>01/19/2026</t>
+          <t>02/09/2026</t>
         </is>
       </c>
       <c r="L11" s="9" t="n">
-        <v>3217146</v>
+        <v>4224158</v>
       </c>
       <c r="M11" s="9" t="inlineStr">
         <is>
@@ -25079,12 +25018,12 @@
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>265250746232</t>
+          <t>253174349440</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>HARPURA TRANS INC</t>
+          <t>HANDSOME TRANSPORTATION INC</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
@@ -25093,7 +25032,7 @@
         </is>
       </c>
       <c r="D12" s="8" t="n">
-        <v>220864.42</v>
+        <v>548010.52</v>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
@@ -25101,7 +25040,7 @@
         </is>
       </c>
       <c r="F12" s="7" t="n">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
@@ -25110,26 +25049,26 @@
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>Reliance Partners, LLC</t>
+          <t>Safeline Insurance Agency, Inc.</t>
         </is>
       </c>
       <c r="I12" s="7" t="inlineStr">
         <is>
-          <t>Daven Loomba</t>
+          <t>Gohar Aramyan</t>
         </is>
       </c>
       <c r="J12" s="7" t="inlineStr">
         <is>
-          <t>04/08/2026</t>
+          <t>08/18/2025</t>
         </is>
       </c>
       <c r="K12" s="7" t="inlineStr">
         <is>
-          <t>01/09/2026</t>
+          <t>01/19/2026</t>
         </is>
       </c>
       <c r="L12" s="7" t="n">
-        <v>3824834</v>
+        <v>3217146</v>
       </c>
       <c r="M12" s="7" t="inlineStr">
         <is>
@@ -25140,12 +25079,12 @@
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
         <is>
-          <t>257630773143</t>
+          <t>265250746232</t>
         </is>
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>EJG TRUCKING INC</t>
+          <t>HARPURA TRANS INC</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
@@ -25154,7 +25093,7 @@
         </is>
       </c>
       <c r="D13" s="10" t="n">
-        <v>144665.42</v>
+        <v>220864.42</v>
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
@@ -25162,7 +25101,7 @@
         </is>
       </c>
       <c r="F13" s="9" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
@@ -25171,42 +25110,42 @@
       </c>
       <c r="H13" s="9" t="inlineStr">
         <is>
-          <t>Saint George Insurance Brokerage, Inc.</t>
+          <t>Reliance Partners, LLC</t>
         </is>
       </c>
       <c r="I13" s="9" t="inlineStr">
         <is>
-          <t>Bethany Bray</t>
+          <t>Daven Loomba</t>
         </is>
       </c>
       <c r="J13" s="9" t="inlineStr">
         <is>
-          <t>06/17/2025</t>
+          <t>04/08/2026</t>
         </is>
       </c>
       <c r="K13" s="9" t="inlineStr">
         <is>
-          <t>02/09/2026</t>
+          <t>01/09/2026</t>
         </is>
       </c>
       <c r="L13" s="9" t="n">
-        <v>3846475</v>
+        <v>3824834</v>
       </c>
       <c r="M13" s="9" t="inlineStr">
         <is>
-          <t>dash_cam_dual_ai_connected</t>
+          <t>eld_only</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>257718771651</t>
+          <t>257630773143</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>NEURON TRANS INC</t>
+          <t>EJG TRUCKING INC</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
@@ -25215,7 +25154,7 @@
         </is>
       </c>
       <c r="D14" s="8" t="n">
-        <v>133698.34</v>
+        <v>144665.42</v>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
@@ -25223,51 +25162,51 @@
         </is>
       </c>
       <c r="F14" s="7" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>Jagdeep Singh Insurance Agency, Inc</t>
+          <t>Saint George Insurance Brokerage, Inc.</t>
         </is>
       </c>
       <c r="I14" s="7" t="inlineStr">
         <is>
-          <t>ARUNDEEP SINGH</t>
+          <t>Bethany Bray</t>
         </is>
       </c>
       <c r="J14" s="7" t="inlineStr">
         <is>
-          <t>06/05/2025</t>
+          <t>06/17/2025</t>
         </is>
       </c>
       <c r="K14" s="7" t="inlineStr">
         <is>
-          <t>01/28/2026</t>
+          <t>02/09/2026</t>
         </is>
       </c>
       <c r="L14" s="7" t="n">
-        <v>4043008</v>
+        <v>3846475</v>
       </c>
       <c r="M14" s="7" t="inlineStr">
         <is>
-          <t>eld_only</t>
+          <t>dash_cam_dual_ai_connected</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>261309376885</t>
+          <t>257718771651</t>
         </is>
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>EAGLE TRANSIT INC</t>
+          <t>NEURON TRANS INC</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
@@ -25276,7 +25215,7 @@
         </is>
       </c>
       <c r="D15" s="10" t="n">
-        <v>107958.34</v>
+        <v>133698.34</v>
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
@@ -25284,11 +25223,11 @@
         </is>
       </c>
       <c r="F15" s="9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G15" s="9" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="H15" s="9" t="inlineStr">
@@ -25298,21 +25237,21 @@
       </c>
       <c r="I15" s="9" t="inlineStr">
         <is>
-          <t>Ateetpal Bansal</t>
+          <t>ARUNDEEP SINGH</t>
         </is>
       </c>
       <c r="J15" s="9" t="inlineStr">
         <is>
-          <t>05/23/2026</t>
+          <t>06/05/2025</t>
         </is>
       </c>
       <c r="K15" s="9" t="inlineStr">
         <is>
-          <t>02/23/2026</t>
+          <t>01/28/2026</t>
         </is>
       </c>
       <c r="L15" s="9" t="n">
-        <v>3455753</v>
+        <v>4043008</v>
       </c>
       <c r="M15" s="9" t="inlineStr">
         <is>
@@ -25323,12 +25262,12 @@
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>263542089381</t>
+          <t>261309376885</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>ADV TRUCKING LLC</t>
+          <t>EAGLE TRANSIT INC</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
@@ -25337,7 +25276,7 @@
         </is>
       </c>
       <c r="D16" s="8" t="n">
-        <v>101099.3</v>
+        <v>107958.34</v>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
@@ -25349,31 +25288,31 @@
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>Empire Company Insurance Services, Inc.</t>
+          <t>Jagdeep Singh Insurance Agency, Inc</t>
         </is>
       </c>
       <c r="I16" s="7" t="inlineStr">
         <is>
-          <t>Jennifer Reimers</t>
+          <t>Ateetpal Bansal</t>
         </is>
       </c>
       <c r="J16" s="7" t="inlineStr">
         <is>
-          <t>06/03/2026</t>
+          <t>05/23/2026</t>
         </is>
       </c>
       <c r="K16" s="7" t="inlineStr">
         <is>
-          <t>03/06/2026</t>
+          <t>02/23/2026</t>
         </is>
       </c>
       <c r="L16" s="7" t="n">
-        <v>2070108</v>
+        <v>3455753</v>
       </c>
       <c r="M16" s="7" t="inlineStr">
         <is>
@@ -25764,7 +25703,7 @@
         </is>
       </c>
       <c r="D23" s="10" t="n">
-        <v>4277.76</v>
+        <v>4796.4</v>
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
@@ -25772,7 +25711,7 @@
         </is>
       </c>
       <c r="F23" s="9" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G23" s="9" t="inlineStr">
         <is>

</xml_diff>